<commit_message>
scan: seg4 2026-06-23 00:03 CST
</commit_message>
<xml_diff>
--- a/output/full_scan/batch_seq5_2026-06-22.xlsx
+++ b/output/full_scan/batch_seq5_2026-06-22.xlsx
@@ -552,10 +552,10 @@
         <v>0</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>69.61029065558286</v>
+        <v>69.61029064531715</v>
       </c>
       <c r="I2" s="2" t="n">
-        <v>23.34902371690885</v>
+        <v>23.34902367880133</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>1.791268981321908</v>
@@ -570,7 +570,7 @@
         <v>-1</v>
       </c>
       <c r="N2" s="2" t="n">
-        <v>1.8595137144464</v>
+        <v>1.85951371465241</v>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
@@ -605,10 +605,10 @@
         <v>0</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>70.52410215444991</v>
+        <v>70.52410216043037</v>
       </c>
       <c r="I3" s="2" t="n">
-        <v>36.98777681077515</v>
+        <v>36.98777681942261</v>
       </c>
       <c r="J3" s="2" t="n">
         <v>1.066569853336768</v>
@@ -623,7 +623,7 @@
         <v>-1</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>0.8896879438036462</v>
+        <v>0.8896879439272882</v>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
@@ -658,10 +658,10 @@
         <v>0</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>61.56247749460944</v>
+        <v>61.56247745942223</v>
       </c>
       <c r="I4" s="2" t="n">
-        <v>15.02158278695572</v>
+        <v>15.02158276477504</v>
       </c>
       <c r="J4" s="2" t="n">
         <v>2.968701240726407</v>
@@ -676,7 +676,7 @@
         <v>-1</v>
       </c>
       <c r="N4" s="2" t="n">
-        <v>0.7477299786190339</v>
+        <v>0.7477299787941811</v>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
@@ -711,10 +711,10 @@
         <v>0</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>63.16863392024053</v>
+        <v>63.16863376087127</v>
       </c>
       <c r="I5" s="2" t="n">
-        <v>17.28187005825511</v>
+        <v>17.28187004663687</v>
       </c>
       <c r="J5" s="2" t="n">
         <v>2.251411393795782</v>
@@ -729,7 +729,7 @@
         <v>-1</v>
       </c>
       <c r="N5" s="2" t="n">
-        <v>0.4212956533123936</v>
+        <v>0.4212956538275281</v>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
@@ -764,10 +764,10 @@
         <v>0</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>63.23248954939959</v>
+        <v>63.2324895232299</v>
       </c>
       <c r="I6" s="2" t="n">
-        <v>15.58513021253922</v>
+        <v>15.5851301915046</v>
       </c>
       <c r="J6" s="2" t="n">
         <v>5.239715494941074</v>
@@ -782,7 +782,7 @@
         <v>-1</v>
       </c>
       <c r="N6" s="2" t="n">
-        <v>0.0561633067327831</v>
+        <v>0.0561633068152065</v>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
@@ -817,10 +817,10 @@
         <v>0</v>
       </c>
       <c r="H7" s="2" t="n">
-        <v>65.79491151341092</v>
+        <v>65.79491147740529</v>
       </c>
       <c r="I7" s="2" t="n">
-        <v>27.56923406016836</v>
+        <v>27.5692340207598</v>
       </c>
       <c r="J7" s="2" t="n">
         <v>1.524268259580351</v>
@@ -835,7 +835,7 @@
         <v>-1</v>
       </c>
       <c r="N7" s="2" t="n">
-        <v>0.8196506801941899</v>
+        <v>0.8196506803281203</v>
       </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
@@ -870,10 +870,10 @@
         <v>0</v>
       </c>
       <c r="H8" s="2" t="n">
-        <v>61.75125425400217</v>
+        <v>61.75125426204967</v>
       </c>
       <c r="I8" s="2" t="n">
-        <v>20.54664773612168</v>
+        <v>20.54664779513035</v>
       </c>
       <c r="J8" s="2" t="n">
         <v>0.8373959422513586</v>
@@ -888,7 +888,7 @@
         <v>-1</v>
       </c>
       <c r="N8" s="2" t="n">
-        <v>40.63120707692542</v>
+        <v>40.63120706868472</v>
       </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
@@ -923,10 +923,10 @@
         <v>0</v>
       </c>
       <c r="H9" s="2" t="n">
-        <v>62.06725739121525</v>
+        <v>62.0672573890572</v>
       </c>
       <c r="I9" s="2" t="n">
-        <v>24.52383627604301</v>
+        <v>24.52383617723065</v>
       </c>
       <c r="J9" s="2" t="n">
         <v>0.5986766579851636</v>
@@ -941,7 +941,7 @@
         <v>-1</v>
       </c>
       <c r="N9" s="2" t="n">
-        <v>0.6657460365676986</v>
+        <v>0.6657460367119477</v>
       </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
@@ -976,10 +976,10 @@
         <v>0</v>
       </c>
       <c r="H10" s="2" t="n">
-        <v>73.49525723338863</v>
+        <v>73.4952572254607</v>
       </c>
       <c r="I10" s="2" t="n">
-        <v>46.87073590428158</v>
+        <v>46.87073597497658</v>
       </c>
       <c r="J10" s="2" t="n">
         <v>1.988780137774658</v>
@@ -994,7 +994,7 @@
         <v>-1</v>
       </c>
       <c r="N10" s="2" t="n">
-        <v>-0.1905508312008894</v>
+        <v>-0.1905508311184736</v>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
@@ -1029,10 +1029,10 @@
         <v>0</v>
       </c>
       <c r="H11" s="2" t="n">
-        <v>59.08547832605755</v>
+        <v>59.08547836126192</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>18.52527998978096</v>
+        <v>18.52528008893096</v>
       </c>
       <c r="J11" s="2" t="n">
         <v>1.560632040710034</v>
@@ -1047,7 +1047,7 @@
         <v>-1</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>0.4774063165070963</v>
+        <v>0.47740631702221</v>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
@@ -1082,10 +1082,10 @@
         <v>0</v>
       </c>
       <c r="H12" s="2" t="n">
-        <v>67.32486951395444</v>
+        <v>67.32486948885929</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>32.77960534676097</v>
+        <v>32.77960537496086</v>
       </c>
       <c r="J12" s="2" t="n">
         <v>0.4922448128066007</v>
@@ -1100,7 +1100,7 @@
         <v>-1</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>13.29684393532084</v>
+        <v>13.29684393748458</v>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
@@ -1135,10 +1135,10 @@
         <v>0</v>
       </c>
       <c r="H13" s="2" t="n">
-        <v>70.66337048685185</v>
+        <v>70.66337046534157</v>
       </c>
       <c r="I13" s="2" t="n">
-        <v>34.93776192974087</v>
+        <v>34.93776189549411</v>
       </c>
       <c r="J13" s="2" t="n">
         <v>1.65976086999231</v>
@@ -1153,7 +1153,7 @@
         <v>-1</v>
       </c>
       <c r="N13" s="2" t="n">
-        <v>0.9828426969592892</v>
+        <v>0.9828426970314136</v>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
@@ -1188,10 +1188,10 @@
         <v>0</v>
       </c>
       <c r="H14" s="2" t="n">
-        <v>70.52804613890115</v>
+        <v>70.52804604647392</v>
       </c>
       <c r="I14" s="2" t="n">
-        <v>26.90513864009864</v>
+        <v>26.90513874293611</v>
       </c>
       <c r="J14" s="2" t="n">
         <v>1.888225466442897</v>
@@ -1206,7 +1206,7 @@
         <v>-1</v>
       </c>
       <c r="N14" s="2" t="n">
-        <v>0.3856330937557957</v>
+        <v>0.3856330939927631</v>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
@@ -1241,10 +1241,10 @@
         <v>0</v>
       </c>
       <c r="H15" s="2" t="n">
-        <v>69.10322023239041</v>
+        <v>69.10322020537672</v>
       </c>
       <c r="I15" s="2" t="n">
-        <v>20.81437179962403</v>
+        <v>20.81437165925641</v>
       </c>
       <c r="J15" s="2" t="n">
         <v>1.469732572659521</v>
@@ -1259,7 +1259,7 @@
         <v>-1</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>0.6582677085161288</v>
+        <v>0.6582677090415889</v>
       </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
@@ -1294,10 +1294,10 @@
         <v>0</v>
       </c>
       <c r="H16" s="2" t="n">
-        <v>68.84524354169626</v>
+        <v>68.84524356899749</v>
       </c>
       <c r="I16" s="2" t="n">
-        <v>35.04716959521522</v>
+        <v>35.04716962007633</v>
       </c>
       <c r="J16" s="2" t="n">
         <v>3.170230799868466</v>
@@ -1312,7 +1312,7 @@
         <v>-1</v>
       </c>
       <c r="N16" s="2" t="n">
-        <v>0.1512263140777068</v>
+        <v>0.1512263140983125</v>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
@@ -1350,7 +1350,7 @@
         <v>73.40712482947494</v>
       </c>
       <c r="I17" s="2" t="n">
-        <v>35.65462944657558</v>
+        <v>35.65462937720459</v>
       </c>
       <c r="J17" s="2" t="n">
         <v>0.1478963673387946</v>
@@ -1365,7 +1365,7 @@
         <v>-1</v>
       </c>
       <c r="N17" s="2" t="n">
-        <v>1.599784518952168</v>
+        <v>1.599784519044888</v>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
@@ -1400,10 +1400,10 @@
         <v>0</v>
       </c>
       <c r="H18" s="2" t="n">
-        <v>63.42604756105855</v>
+        <v>63.42604751646444</v>
       </c>
       <c r="I18" s="2" t="n">
-        <v>28.61559031858852</v>
+        <v>28.61559029222401</v>
       </c>
       <c r="J18" s="2" t="n">
         <v>1.023122487844372</v>
@@ -1418,7 +1418,7 @@
         <v>-1</v>
       </c>
       <c r="N18" s="2" t="n">
-        <v>2.139303881620456</v>
+        <v>2.139303882547733</v>
       </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
@@ -1439,7 +1439,7 @@
         <v/>
       </c>
       <c r="D19" s="2" t="n">
-        <v>922.475621714492</v>
+        <v>922.4756217144908</v>
       </c>
       <c r="E19" s="2" t="n">
         <v>29.6</v>
@@ -1453,10 +1453,10 @@
         <v>0</v>
       </c>
       <c r="H19" s="2" t="n">
-        <v>67.24998777232008</v>
+        <v>67.24998763425936</v>
       </c>
       <c r="I19" s="2" t="n">
-        <v>33.34329473113482</v>
+        <v>33.34329476006803</v>
       </c>
       <c r="J19" s="2" t="n">
         <v>1.566286486227084</v>
@@ -1471,7 +1471,7 @@
         <v>-1</v>
       </c>
       <c r="N19" s="2" t="n">
-        <v>0.1785803221440757</v>
+        <v>0.1785803225767961</v>
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
@@ -1492,7 +1492,7 @@
         <v/>
       </c>
       <c r="D20" s="2" t="n">
-        <v>921.4965700861602</v>
+        <v>921.4965700861604</v>
       </c>
       <c r="E20" s="2" t="n">
         <v>35.55</v>
@@ -1506,10 +1506,10 @@
         <v>0</v>
       </c>
       <c r="H20" s="2" t="n">
-        <v>57.63448923679835</v>
+        <v>57.63448921308942</v>
       </c>
       <c r="I20" s="2" t="n">
-        <v>8.954132051259288</v>
+        <v>8.954132125791702</v>
       </c>
       <c r="J20" s="2" t="n">
         <v>1.218042446083362</v>
@@ -1524,7 +1524,7 @@
         <v>-1</v>
       </c>
       <c r="N20" s="2" t="n">
-        <v>0.1253630345770802</v>
+        <v>0.1253630347316201</v>
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
@@ -1559,10 +1559,10 @@
         <v>0</v>
       </c>
       <c r="H21" s="2" t="n">
-        <v>58.70429302146425</v>
+        <v>58.70429294891465</v>
       </c>
       <c r="I21" s="2" t="n">
-        <v>24.25890970481967</v>
+        <v>24.25890973500521</v>
       </c>
       <c r="J21" s="2" t="n">
         <v>1.359228804072761</v>
@@ -1577,7 +1577,7 @@
         <v>-1</v>
       </c>
       <c r="N21" s="2" t="n">
-        <v>-0.024131481141648</v>
+        <v>-0.0241314804204655</v>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
@@ -1612,10 +1612,10 @@
         <v>0</v>
       </c>
       <c r="H22" s="2" t="n">
-        <v>70.05345144836822</v>
+        <v>70.05345143604127</v>
       </c>
       <c r="I22" s="2" t="n">
-        <v>13.40721369080739</v>
+        <v>13.40721371733455</v>
       </c>
       <c r="J22" s="2" t="n">
         <v>6.234808493472712</v>
@@ -1630,7 +1630,7 @@
         <v>-1</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>0.1308278031198089</v>
+        <v>0.1308278031404143</v>
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
@@ -1665,10 +1665,10 @@
         <v>0</v>
       </c>
       <c r="H23" s="2" t="n">
-        <v>82.49001219176618</v>
+        <v>82.49001217207154</v>
       </c>
       <c r="I23" s="2" t="n">
-        <v>40.5116426887348</v>
+        <v>40.51164259805513</v>
       </c>
       <c r="J23" s="2" t="n">
         <v>1.168056761999391</v>
@@ -1683,7 +1683,7 @@
         <v>-1</v>
       </c>
       <c r="N23" s="2" t="n">
-        <v>1.434924950742543</v>
+        <v>1.434924950835272</v>
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
@@ -1704,7 +1704,7 @@
         <v/>
       </c>
       <c r="D24" s="2" t="n">
-        <v>868.8099423459912</v>
+        <v>868.8099423459906</v>
       </c>
       <c r="E24" s="2" t="n">
         <v>267</v>
@@ -1718,10 +1718,10 @@
         <v>0</v>
       </c>
       <c r="H24" s="2" t="n">
-        <v>63.58766631361207</v>
+        <v>63.58766629040977</v>
       </c>
       <c r="I24" s="2" t="n">
-        <v>32.42480802992792</v>
+        <v>32.42480789428689</v>
       </c>
       <c r="J24" s="2" t="n">
         <v>0.5995684029743191</v>
@@ -1736,7 +1736,7 @@
         <v>-1</v>
       </c>
       <c r="N24" s="2" t="n">
-        <v>-1.010491004130998</v>
+        <v>-1.010491002606159</v>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
@@ -1774,7 +1774,7 @@
         <v>62.7355098534816</v>
       </c>
       <c r="I25" s="2" t="n">
-        <v>29.36996128485517</v>
+        <v>29.36996122055972</v>
       </c>
       <c r="J25" s="2" t="n">
         <v>0.5280129256236559</v>
@@ -1789,7 +1789,7 @@
         <v>-1</v>
       </c>
       <c r="N25" s="2" t="n">
-        <v>-0.00391482416887</v>
+        <v>-0.0039148242718987</v>
       </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
@@ -1824,10 +1824,10 @@
         <v>0</v>
       </c>
       <c r="H26" s="2" t="n">
-        <v>65.92964481926279</v>
+        <v>65.92964473054673</v>
       </c>
       <c r="I26" s="2" t="n">
-        <v>39.70671164908181</v>
+        <v>39.70671163853476</v>
       </c>
       <c r="J26" s="2" t="n">
         <v>1.768666927578058</v>
@@ -1842,7 +1842,7 @@
         <v>-1</v>
       </c>
       <c r="N26" s="2" t="n">
-        <v>0.9102781743384634</v>
+        <v>0.9102781746269442</v>
       </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
@@ -1877,10 +1877,10 @@
         <v>0</v>
       </c>
       <c r="H27" s="2" t="n">
-        <v>59.75401678794751</v>
+        <v>59.75401678137213</v>
       </c>
       <c r="I27" s="2" t="n">
-        <v>25.19237435800272</v>
+        <v>25.19237434260878</v>
       </c>
       <c r="J27" s="2" t="n">
         <v>0.6881919073950612</v>
@@ -1895,7 +1895,7 @@
         <v>-1</v>
       </c>
       <c r="N27" s="2" t="n">
-        <v>-6.576530126938394</v>
+        <v>-6.576530126629393</v>
       </c>
       <c r="O27" s="2" t="inlineStr">
         <is>
@@ -1930,10 +1930,10 @@
         <v>0</v>
       </c>
       <c r="H28" s="2" t="n">
-        <v>75.04460996962706</v>
+        <v>75.04460993573005</v>
       </c>
       <c r="I28" s="2" t="n">
-        <v>20.77472349775958</v>
+        <v>20.77472360480709</v>
       </c>
       <c r="J28" s="2" t="n">
         <v>0.7871232777057307</v>
@@ -1948,7 +1948,7 @@
         <v>-1</v>
       </c>
       <c r="N28" s="2" t="n">
-        <v>1.408690995353939</v>
+        <v>1.408690995436358</v>
       </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
@@ -1986,7 +1986,7 @@
         <v>65.50472569950628</v>
       </c>
       <c r="I29" s="2" t="n">
-        <v>26.97286672207873</v>
+        <v>26.97286671455887</v>
       </c>
       <c r="J29" s="2" t="n">
         <v>1.527539833650121</v>
@@ -2001,7 +2001,7 @@
         <v>-1</v>
       </c>
       <c r="N29" s="2" t="n">
-        <v>0.2115877298302185</v>
+        <v>0.2115877298467035</v>
       </c>
       <c r="O29" s="2" t="inlineStr">
         <is>
@@ -2036,10 +2036,10 @@
         <v>0</v>
       </c>
       <c r="H30" s="2" t="n">
-        <v>58.48397462394407</v>
+        <v>58.48397454673017</v>
       </c>
       <c r="I30" s="2" t="n">
-        <v>13.69330337345906</v>
+        <v>13.69330333887754</v>
       </c>
       <c r="J30" s="2" t="n">
         <v>2.121170525515699</v>
@@ -2054,7 +2054,7 @@
         <v>-1</v>
       </c>
       <c r="N30" s="2" t="n">
-        <v>0.1873089768062046</v>
+        <v>0.187308976868037</v>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
@@ -2092,7 +2092,7 @@
         <v>65.17486382832099</v>
       </c>
       <c r="I31" s="2" t="n">
-        <v>13.9130124280457</v>
+        <v>13.91301243309399</v>
       </c>
       <c r="J31" s="2" t="n">
         <v>0.5145015808727416</v>
@@ -2107,7 +2107,7 @@
         <v>-1</v>
       </c>
       <c r="N31" s="2" t="n">
-        <v>1.461306849392056</v>
+        <v>1.461306849144799</v>
       </c>
       <c r="O31" s="2" t="inlineStr">
         <is>
@@ -2142,10 +2142,10 @@
         <v>0</v>
       </c>
       <c r="H32" s="2" t="n">
-        <v>62.98429936672268</v>
+        <v>62.98429931552152</v>
       </c>
       <c r="I32" s="2" t="n">
-        <v>27.34986544416343</v>
+        <v>27.34986536882829</v>
       </c>
       <c r="J32" s="2" t="n">
         <v>0.708073961153506</v>
@@ -2160,7 +2160,7 @@
         <v>-1</v>
       </c>
       <c r="N32" s="2" t="n">
-        <v>-0.0604413131533813</v>
+        <v>-0.0604413131121693</v>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
@@ -2195,10 +2195,10 @@
         <v>0</v>
       </c>
       <c r="H33" s="2" t="n">
-        <v>67.67391242185673</v>
+        <v>67.67391241325376</v>
       </c>
       <c r="I33" s="2" t="n">
-        <v>45.46503903062371</v>
+        <v>45.46503906185094</v>
       </c>
       <c r="J33" s="2" t="n">
         <v>1.37464952542939</v>
@@ -2213,7 +2213,7 @@
         <v>-1</v>
       </c>
       <c r="N33" s="2" t="n">
-        <v>-0.4325190953327071</v>
+        <v>-0.4325190952193729</v>
       </c>
       <c r="O33" s="2" t="inlineStr">
         <is>
@@ -2248,10 +2248,10 @@
         <v>0</v>
       </c>
       <c r="H34" s="2" t="n">
-        <v>66.78587757341214</v>
+        <v>66.78587755738536</v>
       </c>
       <c r="I34" s="2" t="n">
-        <v>35.22890096347807</v>
+        <v>35.22890093847078</v>
       </c>
       <c r="J34" s="2" t="n">
         <v>2.269905627035785</v>
@@ -2266,7 +2266,7 @@
         <v>-1</v>
       </c>
       <c r="N34" s="2" t="n">
-        <v>-0.012107211474291</v>
+        <v>-0.012107211453685</v>
       </c>
       <c r="O34" s="2" t="inlineStr">
         <is>
@@ -2287,7 +2287,7 @@
         <v/>
       </c>
       <c r="D35" s="2" t="n">
-        <v>807.1776118907775</v>
+        <v>807.1776118907776</v>
       </c>
       <c r="E35" s="2" t="n">
         <v>118</v>
@@ -2301,10 +2301,10 @@
         <v>0</v>
       </c>
       <c r="H35" s="2" t="n">
-        <v>57.18310780638964</v>
+        <v>57.18310763025012</v>
       </c>
       <c r="I35" s="2" t="n">
-        <v>14.99679776572183</v>
+        <v>14.99679786130617</v>
       </c>
       <c r="J35" s="2" t="n">
         <v>1.416461069533455</v>
@@ -2319,7 +2319,7 @@
         <v>-1</v>
       </c>
       <c r="N35" s="2" t="n">
-        <v>0.4255205874532903</v>
+        <v>0.4255205880714798</v>
       </c>
       <c r="O35" s="2" t="inlineStr">
         <is>
@@ -2354,10 +2354,10 @@
         <v>0</v>
       </c>
       <c r="H36" s="2" t="n">
-        <v>60.98744468826789</v>
+        <v>60.98744463218766</v>
       </c>
       <c r="I36" s="2" t="n">
-        <v>59.59776614802397</v>
+        <v>59.59776610909118</v>
       </c>
       <c r="J36" s="2" t="n">
         <v>0.3638457579178084</v>
@@ -2372,7 +2372,7 @@
         <v>-1</v>
       </c>
       <c r="N36" s="2" t="n">
-        <v>-0.1902824975569348</v>
+        <v>-0.1902824974333028</v>
       </c>
       <c r="O36" s="2" t="inlineStr">
         <is>
@@ -2407,10 +2407,10 @@
         <v>0</v>
       </c>
       <c r="H37" s="2" t="n">
-        <v>67.34350042599064</v>
+        <v>67.34350042676955</v>
       </c>
       <c r="I37" s="2" t="n">
-        <v>32.57523094651178</v>
+        <v>32.57523093873085</v>
       </c>
       <c r="J37" s="2" t="n">
         <v>1.209495769291389</v>
@@ -2425,7 +2425,7 @@
         <v>-1</v>
       </c>
       <c r="N37" s="2" t="n">
-        <v>6.267028561659302</v>
+        <v>6.267028561679922</v>
       </c>
       <c r="O37" s="2" t="inlineStr">
         <is>
@@ -2460,10 +2460,10 @@
         <v>0</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>54.36987125364193</v>
+        <v>54.36987120726562</v>
       </c>
       <c r="I38" s="2" t="n">
-        <v>29.35067459022847</v>
+        <v>29.3506745816252</v>
       </c>
       <c r="J38" s="2" t="n">
         <v>0.6372237154001658</v>
@@ -2478,7 +2478,7 @@
         <v>-1</v>
       </c>
       <c r="N38" s="2" t="n">
-        <v>-0.3562925108126413</v>
+        <v>-0.3562925107472452</v>
       </c>
       <c r="O38" s="2" t="inlineStr">
         <is>
@@ -2513,10 +2513,10 @@
         <v>0</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>59.26134815597292</v>
+        <v>59.26134791905825</v>
       </c>
       <c r="I39" s="2" t="n">
-        <v>16.73019221719993</v>
+        <v>16.73019210144061</v>
       </c>
       <c r="J39" s="2" t="n">
         <v>0.7829770262135554</v>
@@ -2531,7 +2531,7 @@
         <v>-1</v>
       </c>
       <c r="N39" s="2" t="n">
-        <v>0.0353051103133304</v>
+        <v>0.0353051106841355</v>
       </c>
       <c r="O39" s="2" t="inlineStr">
         <is>
@@ -2566,10 +2566,10 @@
         <v>0</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>55.20246880100045</v>
+        <v>55.20246874320565</v>
       </c>
       <c r="I40" s="2" t="n">
-        <v>26.31987039971836</v>
+        <v>26.31987043884513</v>
       </c>
       <c r="J40" s="2" t="n">
         <v>0.65591067375503</v>
@@ -2584,7 +2584,7 @@
         <v>-1</v>
       </c>
       <c r="N40" s="2" t="n">
-        <v>-0.2193695720133826</v>
+        <v>-0.2193695719000495</v>
       </c>
       <c r="O40" s="2" t="inlineStr">
         <is>
@@ -2622,7 +2622,7 @@
         <v>62.09415151193513</v>
       </c>
       <c r="I41" s="2" t="n">
-        <v>37.07442235731499</v>
+        <v>37.07442239737025</v>
       </c>
       <c r="J41" s="2" t="n">
         <v>0.3956928462558463</v>
@@ -2672,10 +2672,10 @@
         <v>0</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>60.19625835323176</v>
+        <v>60.19625835131896</v>
       </c>
       <c r="I42" s="2" t="n">
-        <v>51.22763587074565</v>
+        <v>51.22763591412657</v>
       </c>
       <c r="J42" s="2" t="n">
         <v>0.8081257960711156</v>
@@ -2690,7 +2690,7 @@
         <v>-1</v>
       </c>
       <c r="N42" s="2" t="n">
-        <v>-0.6859197233740328</v>
+        <v>-0.6859197233637362</v>
       </c>
       <c r="O42" s="2" t="inlineStr">
         <is>
@@ -2711,7 +2711,7 @@
         <v/>
       </c>
       <c r="D43" s="2" t="n">
-        <v>751.3538664019605</v>
+        <v>751.3538664019602</v>
       </c>
       <c r="E43" s="2" t="n">
         <v>156.5</v>
@@ -2725,10 +2725,10 @@
         <v>0</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>65.04745932396852</v>
+        <v>65.04745928251592</v>
       </c>
       <c r="I43" s="2" t="n">
-        <v>19.94458541258645</v>
+        <v>19.94458542961824</v>
       </c>
       <c r="J43" s="2" t="n">
         <v>2.117585244598668</v>
@@ -2778,10 +2778,10 @@
         <v>0</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>67.16317891579266</v>
+        <v>67.16317881724868</v>
       </c>
       <c r="I44" s="2" t="n">
-        <v>22.56888866269279</v>
+        <v>22.56888858597627</v>
       </c>
       <c r="J44" s="2" t="n">
         <v>1.847623159447953</v>
@@ -2796,7 +2796,7 @@
         <v>-1</v>
       </c>
       <c r="N44" s="2" t="n">
-        <v>0.1523015810794318</v>
+        <v>0.1523015811103417</v>
       </c>
       <c r="O44" s="2" t="inlineStr">
         <is>
@@ -2831,10 +2831,10 @@
         <v>0</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>72.92062220761136</v>
+        <v>72.92062220001588</v>
       </c>
       <c r="I45" s="2" t="n">
-        <v>54.69681982385165</v>
+        <v>54.696819769544</v>
       </c>
       <c r="J45" s="2" t="n">
         <v>0.896457088527064</v>
@@ -2849,7 +2849,7 @@
         <v>-1</v>
       </c>
       <c r="N45" s="2" t="n">
-        <v>1.599179246756417</v>
+        <v>1.599179246849154</v>
       </c>
       <c r="O45" s="2" t="inlineStr">
         <is>
@@ -2884,10 +2884,10 @@
         <v>0</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>86.00120896743896</v>
+        <v>86.00120885759905</v>
       </c>
       <c r="I46" s="2" t="n">
-        <v>33.41126891301832</v>
+        <v>33.41126901196995</v>
       </c>
       <c r="J46" s="2" t="n">
         <v>1.151024613034979</v>
@@ -2902,7 +2902,7 @@
         <v>-1</v>
       </c>
       <c r="N46" s="2" t="n">
-        <v>1.083258901333429</v>
+        <v>1.083258902466744</v>
       </c>
       <c r="O46" s="2" t="inlineStr">
         <is>
@@ -2937,10 +2937,10 @@
         <v>0</v>
       </c>
       <c r="H47" s="2" t="n">
-        <v>66.8323286668672</v>
+        <v>66.83232864847196</v>
       </c>
       <c r="I47" s="2" t="n">
-        <v>29.18715686874278</v>
+        <v>29.18715688857407</v>
       </c>
       <c r="J47" s="2" t="n">
         <v>1.736018235639919</v>
@@ -2955,7 +2955,7 @@
         <v>-1</v>
       </c>
       <c r="N47" s="2" t="n">
-        <v>0.4689050450545609</v>
+        <v>0.4689050450957692</v>
       </c>
       <c r="O47" s="2" t="inlineStr">
         <is>
@@ -2976,7 +2976,7 @@
         <v/>
       </c>
       <c r="D48" s="2" t="n">
-        <v>702.1348559451001</v>
+        <v>702.1348559451</v>
       </c>
       <c r="E48" s="2" t="n">
         <v>22.75</v>
@@ -2990,10 +2990,10 @@
         <v>0</v>
       </c>
       <c r="H48" s="2" t="n">
-        <v>75.95762364610694</v>
+        <v>75.95755407195753</v>
       </c>
       <c r="I48" s="2" t="n">
-        <v>32.90936493723116</v>
+        <v>32.90933544811909</v>
       </c>
       <c r="J48" s="2" t="n">
         <v>2.042545259522813</v>
@@ -3008,7 +3008,7 @@
         <v>-1</v>
       </c>
       <c r="N48" s="2" t="n">
-        <v>0.5271711008087072</v>
+        <v>0.5271711674765165</v>
       </c>
       <c r="O48" s="2" t="inlineStr">
         <is>
@@ -3043,10 +3043,10 @@
         <v>0</v>
       </c>
       <c r="H49" s="2" t="n">
-        <v>49.73714755225461</v>
+        <v>49.73714740207048</v>
       </c>
       <c r="I49" s="2" t="n">
-        <v>21.47835243364892</v>
+        <v>21.47835225980052</v>
       </c>
       <c r="J49" s="2" t="n">
         <v>0.4446543455845625</v>
@@ -3061,7 +3061,7 @@
         <v>-1</v>
       </c>
       <c r="N49" s="2" t="n">
-        <v>-0.5711224590775712</v>
+        <v>-0.5711224582945564</v>
       </c>
       <c r="O49" s="2" t="inlineStr">
         <is>
@@ -3082,7 +3082,7 @@
         <v/>
       </c>
       <c r="D50" s="2" t="n">
-        <v>689.75857727487</v>
+        <v>689.7585772748699</v>
       </c>
       <c r="E50" s="2" t="n">
         <v>39.35</v>
@@ -3096,10 +3096,10 @@
         <v>0</v>
       </c>
       <c r="H50" s="2" t="n">
-        <v>61.23244981436592</v>
+        <v>61.23244979989367</v>
       </c>
       <c r="I50" s="2" t="n">
-        <v>36.12354138063647</v>
+        <v>36.12354133978289</v>
       </c>
       <c r="J50" s="2" t="n">
         <v>0.8447879334847649</v>
@@ -3114,7 +3114,7 @@
         <v>-1</v>
       </c>
       <c r="N50" s="2" t="n">
-        <v>-0.26226656745386</v>
+        <v>-0.2622665672890174</v>
       </c>
       <c r="O50" s="2" t="inlineStr">
         <is>
@@ -3149,10 +3149,10 @@
         <v>0</v>
       </c>
       <c r="H51" s="2" t="n">
-        <v>55.03130527384693</v>
+        <v>55.03130516562817</v>
       </c>
       <c r="I51" s="2" t="n">
-        <v>29.02963258295912</v>
+        <v>29.02963255448561</v>
       </c>
       <c r="J51" s="2" t="n">
         <v>0.7073331945600417</v>
@@ -3167,7 +3167,7 @@
         <v>-1</v>
       </c>
       <c r="N51" s="2" t="n">
-        <v>-0.1834981719485142</v>
+        <v>-0.1834981705061062</v>
       </c>
       <c r="O51" s="2" t="inlineStr">
         <is>
@@ -3202,10 +3202,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="2" t="n">
-        <v>54.51350400280162</v>
+        <v>54.51350399035245</v>
       </c>
       <c r="I52" s="2" t="n">
-        <v>17.90289291615174</v>
+        <v>17.90289285808902</v>
       </c>
       <c r="J52" s="2" t="n">
         <v>0.8499321292406526</v>
@@ -3220,7 +3220,7 @@
         <v>-1</v>
       </c>
       <c r="N52" s="2" t="n">
-        <v>-1.081632681335054</v>
+        <v>-1.081632681252592</v>
       </c>
       <c r="O52" s="2" t="inlineStr">
         <is>
@@ -3255,10 +3255,10 @@
         <v>0</v>
       </c>
       <c r="H53" s="2" t="n">
-        <v>56.5388704515182</v>
+        <v>56.53887035573174</v>
       </c>
       <c r="I53" s="2" t="n">
-        <v>29.14987035092824</v>
+        <v>29.14987020137885</v>
       </c>
       <c r="J53" s="2" t="n">
         <v>0.9675913675404896</v>
@@ -3273,7 +3273,7 @@
         <v>-1</v>
       </c>
       <c r="N53" s="2" t="n">
-        <v>0.0075920376242728</v>
+        <v>0.0075920376654877</v>
       </c>
       <c r="O53" s="2" t="inlineStr">
         <is>
@@ -3311,7 +3311,7 @@
         <v>52.25717944274824</v>
       </c>
       <c r="I54" s="2" t="n">
-        <v>16.48362768743323</v>
+        <v>16.48362765966231</v>
       </c>
       <c r="J54" s="2" t="n">
         <v>0.9743595141777224</v>
@@ -3326,7 +3326,7 @@
         <v>-1</v>
       </c>
       <c r="N54" s="2" t="n">
-        <v>0.5103651443751493</v>
+        <v>0.5103651444163662</v>
       </c>
       <c r="O54" s="2" t="inlineStr">
         <is>
@@ -3361,10 +3361,10 @@
         <v>0</v>
       </c>
       <c r="H55" s="2" t="n">
-        <v>66.36028437045329</v>
+        <v>66.36028436193584</v>
       </c>
       <c r="I55" s="2" t="n">
-        <v>47.76459003799953</v>
+        <v>47.76458999789444</v>
       </c>
       <c r="J55" s="2" t="n">
         <v>0.715341692563656</v>
@@ -3379,7 +3379,7 @@
         <v>-1</v>
       </c>
       <c r="N55" s="2" t="n">
-        <v>-0.409279869921999</v>
+        <v>-0.4092798698292661</v>
       </c>
       <c r="O55" s="2" t="inlineStr">
         <is>
@@ -3414,10 +3414,10 @@
         <v>0</v>
       </c>
       <c r="H56" s="2" t="n">
-        <v>55.06266438614394</v>
+        <v>55.06266372406642</v>
       </c>
       <c r="I56" s="2" t="n">
-        <v>23.90739844128268</v>
+        <v>23.90739810525046</v>
       </c>
       <c r="J56" s="2" t="n">
         <v>0.750864911342356</v>
@@ -3467,10 +3467,10 @@
         <v>0</v>
       </c>
       <c r="H57" s="2" t="n">
-        <v>51.27125413842486</v>
+        <v>51.27125413801214</v>
       </c>
       <c r="I57" s="2" t="n">
-        <v>21.64434846676498</v>
+        <v>21.64434842041522</v>
       </c>
       <c r="J57" s="2" t="n">
         <v>1.039859771586611</v>
@@ -3506,7 +3506,7 @@
         <v/>
       </c>
       <c r="D58" s="2" t="n">
-        <v>633.9165491666706</v>
+        <v>633.9165491666707</v>
       </c>
       <c r="E58" s="2" t="n">
         <v>108</v>
@@ -3520,10 +3520,10 @@
         <v>0</v>
       </c>
       <c r="H58" s="2" t="n">
-        <v>64.71178105943341</v>
+        <v>64.71178099415988</v>
       </c>
       <c r="I58" s="2" t="n">
-        <v>38.64289792753357</v>
+        <v>38.6428979481167</v>
       </c>
       <c r="J58" s="2" t="n">
         <v>3.07920957139084</v>
@@ -3538,7 +3538,7 @@
         <v>-1</v>
       </c>
       <c r="N58" s="2" t="n">
-        <v>0.5354214992456847</v>
+        <v>0.5354214994723456</v>
       </c>
       <c r="O58" s="2" t="inlineStr">
         <is>
@@ -3573,10 +3573,10 @@
         <v>0</v>
       </c>
       <c r="H59" s="2" t="n">
-        <v>56.20779529832454</v>
+        <v>56.20779526309446</v>
       </c>
       <c r="I59" s="2" t="n">
-        <v>23.51708693134601</v>
+        <v>23.51708701952598</v>
       </c>
       <c r="J59" s="2" t="n">
         <v>2.333996473858205</v>
@@ -3591,7 +3591,7 @@
         <v>-1</v>
       </c>
       <c r="N59" s="2" t="n">
-        <v>0.5094118513502668</v>
+        <v>0.5094118512472479</v>
       </c>
       <c r="O59" s="2" t="inlineStr">
         <is>
@@ -3626,10 +3626,10 @@
         <v>0</v>
       </c>
       <c r="H60" s="2" t="n">
-        <v>58.19527915761321</v>
+        <v>58.19527929747429</v>
       </c>
       <c r="I60" s="2" t="n">
-        <v>21.36578895609528</v>
+        <v>21.3657889675534</v>
       </c>
       <c r="J60" s="2" t="n">
         <v>1.601694407578518</v>
@@ -3644,7 +3644,7 @@
         <v>-1</v>
       </c>
       <c r="N60" s="2" t="n">
-        <v>-0.09091343840077119</v>
+        <v>-0.09091343847289191</v>
       </c>
       <c r="O60" s="2" t="inlineStr">
         <is>
@@ -3665,7 +3665,7 @@
         <v/>
       </c>
       <c r="D61" s="2" t="n">
-        <v>607.8033174102164</v>
+        <v>607.803317410216</v>
       </c>
       <c r="E61" s="2" t="n">
         <v>15.9</v>
@@ -3679,10 +3679,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="2" t="n">
-        <v>61.22594693879771</v>
+        <v>61.22594668010461</v>
       </c>
       <c r="I61" s="2" t="n">
-        <v>29.63111622528217</v>
+        <v>29.63111593283841</v>
       </c>
       <c r="J61" s="2" t="n">
         <v>1.1612697109054</v>
@@ -3697,7 +3697,7 @@
         <v>-1</v>
       </c>
       <c r="N61" s="2" t="n">
-        <v>0.1199235098957916</v>
+        <v>0.1199235101533637</v>
       </c>
       <c r="O61" s="2" t="inlineStr">
         <is>
@@ -3732,10 +3732,10 @@
         <v>0</v>
       </c>
       <c r="H62" s="2" t="n">
-        <v>48.30470430066625</v>
+        <v>48.30470415317998</v>
       </c>
       <c r="I62" s="2" t="n">
-        <v>36.40124488540557</v>
+        <v>36.40124488073397</v>
       </c>
       <c r="J62" s="2" t="n">
         <v>0.3801850840597383</v>
@@ -3750,7 +3750,7 @@
         <v>-1</v>
       </c>
       <c r="N62" s="2" t="n">
-        <v>-1.098102426886505</v>
+        <v>-1.098102426216815</v>
       </c>
       <c r="O62" s="2" t="inlineStr">
         <is>
@@ -3785,10 +3785,10 @@
         <v>0</v>
       </c>
       <c r="H63" s="2" t="n">
-        <v>41.21115847947762</v>
+        <v>41.21115847418831</v>
       </c>
       <c r="I63" s="2" t="n">
-        <v>32.3000315943864</v>
+        <v>32.30003155028481</v>
       </c>
       <c r="J63" s="2" t="n">
         <v>0.8987243358298658</v>
@@ -3803,7 +3803,7 @@
         <v>-1</v>
       </c>
       <c r="N63" s="2" t="n">
-        <v>0.3705161267988526</v>
+        <v>0.3705161268400729</v>
       </c>
       <c r="O63" s="2" t="inlineStr">
         <is>
@@ -3838,10 +3838,10 @@
         <v>0</v>
       </c>
       <c r="H64" s="2" t="n">
-        <v>54.4687240636269</v>
+        <v>54.46872403601537</v>
       </c>
       <c r="I64" s="2" t="n">
-        <v>22.13711546434999</v>
+        <v>22.13711529399873</v>
       </c>
       <c r="J64" s="2" t="n">
         <v>1.12424705556668</v>
@@ -3856,7 +3856,7 @@
         <v>-1</v>
       </c>
       <c r="N64" s="2" t="n">
-        <v>-0.1673959492202277</v>
+        <v>-0.1673959489214351</v>
       </c>
       <c r="O64" s="2" t="inlineStr">
         <is>
@@ -3891,10 +3891,10 @@
         <v>0</v>
       </c>
       <c r="H65" s="2" t="n">
-        <v>54.51240870687316</v>
+        <v>54.51240870352187</v>
       </c>
       <c r="I65" s="2" t="n">
-        <v>14.49193528376961</v>
+        <v>14.49193524023827</v>
       </c>
       <c r="J65" s="2" t="n">
         <v>1.356981481971386</v>
@@ -3909,7 +3909,7 @@
         <v>-1</v>
       </c>
       <c r="N65" s="2" t="n">
-        <v>0.6838836171605623</v>
+        <v>0.6838836171832287</v>
       </c>
       <c r="O65" s="2" t="inlineStr">
         <is>
@@ -3930,7 +3930,7 @@
         <v/>
       </c>
       <c r="D66" s="2" t="n">
-        <v>585.6224555329185</v>
+        <v>585.6224555329184</v>
       </c>
       <c r="E66" s="2" t="n">
         <v>23.55</v>
@@ -3944,10 +3944,10 @@
         <v>0</v>
       </c>
       <c r="H66" s="2" t="n">
-        <v>64.789300960112</v>
+        <v>64.78930090327296</v>
       </c>
       <c r="I66" s="2" t="n">
-        <v>16.85967710869568</v>
+        <v>16.85967717124693</v>
       </c>
       <c r="J66" s="2" t="n">
         <v>1.710481304701167</v>
@@ -3962,7 +3962,7 @@
         <v>-1</v>
       </c>
       <c r="N66" s="2" t="n">
-        <v>0.1262755485462441</v>
+        <v>0.1262755486389692</v>
       </c>
       <c r="O66" s="2" t="inlineStr">
         <is>
@@ -3997,10 +3997,10 @@
         <v>0</v>
       </c>
       <c r="H67" s="2" t="n">
-        <v>54.71268888859277</v>
+        <v>54.71268885490933</v>
       </c>
       <c r="I67" s="2" t="n">
-        <v>36.25557542338299</v>
+        <v>36.25557535572629</v>
       </c>
       <c r="J67" s="2" t="n">
         <v>1.134138480350754</v>
@@ -4015,7 +4015,7 @@
         <v>-1</v>
       </c>
       <c r="N67" s="2" t="n">
-        <v>-3.123514482252089</v>
+        <v>-3.123514481860573</v>
       </c>
       <c r="O67" s="2" t="inlineStr">
         <is>
@@ -4050,10 +4050,10 @@
         <v>0</v>
       </c>
       <c r="H68" s="2" t="n">
-        <v>54.07521111247485</v>
+        <v>54.07521109312209</v>
       </c>
       <c r="I68" s="2" t="n">
-        <v>22.45980791816962</v>
+        <v>22.45980773074209</v>
       </c>
       <c r="J68" s="2" t="n">
         <v>0.8215709577062467</v>
@@ -4068,7 +4068,7 @@
         <v>-1</v>
       </c>
       <c r="N68" s="2" t="n">
-        <v>-7.931924894518648</v>
+        <v>-7.931924893818049</v>
       </c>
       <c r="O68" s="2" t="inlineStr">
         <is>
@@ -4103,10 +4103,10 @@
         <v>0</v>
       </c>
       <c r="H69" s="2" t="n">
-        <v>54.4238230982075</v>
+        <v>54.42382257753046</v>
       </c>
       <c r="I69" s="2" t="n">
-        <v>20.16291601652398</v>
+        <v>20.16291611787561</v>
       </c>
       <c r="J69" s="2" t="n">
         <v>0.4479697303676961</v>
@@ -4121,7 +4121,7 @@
         <v>-1</v>
       </c>
       <c r="N69" s="2" t="n">
-        <v>-0.1301800364139644</v>
+        <v>-0.1301800355897313</v>
       </c>
       <c r="O69" s="2" t="inlineStr">
         <is>
@@ -4156,10 +4156,10 @@
         <v>0</v>
       </c>
       <c r="H70" s="2" t="n">
-        <v>58.89982738481706</v>
+        <v>58.89982735622178</v>
       </c>
       <c r="I70" s="2" t="n">
-        <v>25.56075788263397</v>
+        <v>25.5607578159193</v>
       </c>
       <c r="J70" s="2" t="n">
         <v>0.8313154957006242</v>
@@ -4174,7 +4174,7 @@
         <v>-1</v>
       </c>
       <c r="N70" s="2" t="n">
-        <v>-0.4224226551572998</v>
+        <v>-0.4224226550027565</v>
       </c>
       <c r="O70" s="2" t="inlineStr">
         <is>
@@ -4195,7 +4195,7 @@
         <v/>
       </c>
       <c r="D71" s="2" t="n">
-        <v>553.645044098223</v>
+        <v>553.6450440982229</v>
       </c>
       <c r="E71" s="2" t="n">
         <v>810</v>
@@ -4209,10 +4209,10 @@
         <v>0</v>
       </c>
       <c r="H71" s="2" t="n">
-        <v>54.86271464960051</v>
+        <v>54.86271461812623</v>
       </c>
       <c r="I71" s="2" t="n">
-        <v>22.657797446664</v>
+        <v>22.65779716768054</v>
       </c>
       <c r="J71" s="2" t="n">
         <v>0.7012022631711666</v>
@@ -4227,7 +4227,7 @@
         <v>-1</v>
       </c>
       <c r="N71" s="2" t="n">
-        <v>0.2676628012733353</v>
+        <v>0.2676628040551065</v>
       </c>
       <c r="O71" s="2" t="inlineStr">
         <is>
@@ -4262,10 +4262,10 @@
         <v>0</v>
       </c>
       <c r="H72" s="2" t="n">
-        <v>53.32563123375699</v>
+        <v>53.32563127302051</v>
       </c>
       <c r="I72" s="2" t="n">
-        <v>18.67155085446397</v>
+        <v>18.6715508011213</v>
       </c>
       <c r="J72" s="2" t="n">
         <v>2.176412370373201</v>
@@ -4280,7 +4280,7 @@
         <v>-1</v>
       </c>
       <c r="N72" s="2" t="n">
-        <v>0.0038632648522182</v>
+        <v>0.0038632648934281</v>
       </c>
       <c r="O72" s="2" t="inlineStr">
         <is>
@@ -4315,10 +4315,10 @@
         <v>0</v>
       </c>
       <c r="H73" s="2" t="n">
-        <v>54.16761474391144</v>
+        <v>54.07464430494792</v>
       </c>
       <c r="I73" s="2" t="n">
-        <v>12.9501156807448</v>
+        <v>12.78813456213036</v>
       </c>
       <c r="J73" s="2" t="n">
         <v>0.4265127663271301</v>
@@ -4333,7 +4333,7 @@
         <v>-1</v>
       </c>
       <c r="N73" s="2" t="n">
-        <v>0.5460647822321499</v>
+        <v>0.5464948707817345</v>
       </c>
       <c r="O73" s="2" t="inlineStr">
         <is>
@@ -4368,10 +4368,10 @@
         <v>0</v>
       </c>
       <c r="H74" s="2" t="n">
-        <v>52.48227270157624</v>
+        <v>52.48227262648635</v>
       </c>
       <c r="I74" s="2" t="n">
-        <v>14.90585663348133</v>
+        <v>14.9058565839915</v>
       </c>
       <c r="J74" s="2" t="n">
         <v>0.7374709167287512</v>
@@ -4386,7 +4386,7 @@
         <v>-1</v>
       </c>
       <c r="N74" s="2" t="n">
-        <v>0.0682447066894519</v>
+        <v>0.06824470676157091</v>
       </c>
       <c r="O74" s="2" t="inlineStr">
         <is>
@@ -4421,10 +4421,10 @@
         <v>0</v>
       </c>
       <c r="H75" s="2" t="n">
-        <v>51.88092340338105</v>
+        <v>51.88092332541167</v>
       </c>
       <c r="I75" s="2" t="n">
-        <v>18.13554649579666</v>
+        <v>18.13554631163884</v>
       </c>
       <c r="J75" s="2" t="n">
         <v>0.6096094117955474</v>
@@ -4439,7 +4439,7 @@
         <v>-1</v>
       </c>
       <c r="N75" s="2" t="n">
-        <v>-0.8246468563019396</v>
+        <v>-0.8246468558692164</v>
       </c>
       <c r="O75" s="2" t="inlineStr">
         <is>
@@ -4460,7 +4460,7 @@
         <v/>
       </c>
       <c r="D76" s="2" t="n">
-        <v>542.9887798418403</v>
+        <v>542.9887798418802</v>
       </c>
       <c r="E76" s="2" t="n">
         <v>30.3</v>
@@ -4474,10 +4474,10 @@
         <v>0</v>
       </c>
       <c r="H76" s="2" t="n">
-        <v>53.26546742687465</v>
+        <v>53.26546669483608</v>
       </c>
       <c r="I76" s="2" t="n">
-        <v>29.22660439670638</v>
+        <v>29.22660444190123</v>
       </c>
       <c r="J76" s="2" t="n">
         <v>0.1983414565412168</v>
@@ -4492,7 +4492,7 @@
         <v>-1</v>
       </c>
       <c r="N76" s="2" t="n">
-        <v>-0.0270228732612473</v>
+        <v>-0.0270228722515655</v>
       </c>
       <c r="O76" s="2" t="inlineStr">
         <is>
@@ -4513,7 +4513,7 @@
         <v/>
       </c>
       <c r="D77" s="2" t="n">
-        <v>541.5982771442162</v>
+        <v>541.5982771442161</v>
       </c>
       <c r="E77" s="2" t="n">
         <v>30.65</v>
@@ -4527,10 +4527,10 @@
         <v>0</v>
       </c>
       <c r="H77" s="2" t="n">
-        <v>54.30930108275103</v>
+        <v>54.30930099409608</v>
       </c>
       <c r="I77" s="2" t="n">
-        <v>20.67949439785206</v>
+        <v>20.67949439872461</v>
       </c>
       <c r="J77" s="2" t="n">
         <v>1.74497811530769</v>
@@ -4580,10 +4580,10 @@
         <v>0</v>
       </c>
       <c r="H78" s="2" t="n">
-        <v>48.10753814970104</v>
+        <v>48.10753813037146</v>
       </c>
       <c r="I78" s="2" t="n">
-        <v>9.638516145021775</v>
+        <v>9.638516160816057</v>
       </c>
       <c r="J78" s="2" t="n">
         <v>0.5751802909870444</v>
@@ -4598,7 +4598,7 @@
         <v>-1</v>
       </c>
       <c r="N78" s="2" t="n">
-        <v>-1.098786016187318</v>
+        <v>-1.098786015672178</v>
       </c>
       <c r="O78" s="2" t="inlineStr">
         <is>
@@ -4633,10 +4633,10 @@
         <v>0</v>
       </c>
       <c r="H79" s="2" t="n">
-        <v>52.7338664861217</v>
+        <v>52.73386642916574</v>
       </c>
       <c r="I79" s="2" t="n">
-        <v>18.01879233170907</v>
+        <v>18.01879224858371</v>
       </c>
       <c r="J79" s="2" t="n">
         <v>0.5248147259668191</v>
@@ -4651,7 +4651,7 @@
         <v>-1</v>
       </c>
       <c r="N79" s="2" t="n">
-        <v>-7.752224518739176</v>
+        <v>-7.752224515648269</v>
       </c>
       <c r="O79" s="2" t="inlineStr">
         <is>
@@ -4686,10 +4686,10 @@
         <v>0</v>
       </c>
       <c r="H80" s="2" t="n">
-        <v>54.78525634211037</v>
+        <v>54.78525633100279</v>
       </c>
       <c r="I80" s="2" t="n">
-        <v>27.98284575460833</v>
+        <v>27.98284582260043</v>
       </c>
       <c r="J80" s="2" t="n">
         <v>0.9677256651097508</v>
@@ -4704,7 +4704,7 @@
         <v>-1</v>
       </c>
       <c r="N80" s="2" t="n">
-        <v>0.177225358651547</v>
+        <v>0.1772253586206347</v>
       </c>
       <c r="O80" s="2" t="inlineStr">
         <is>
@@ -4725,7 +4725,7 @@
         <v/>
       </c>
       <c r="D81" s="2" t="n">
-        <v>519.1494343476767</v>
+        <v>519.1494343476766</v>
       </c>
       <c r="E81" s="2" t="n">
         <v>36.8</v>
@@ -4739,10 +4739,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="2" t="n">
-        <v>60.57258457299705</v>
+        <v>60.57258448227383</v>
       </c>
       <c r="I81" s="2" t="n">
-        <v>24.79385102416829</v>
+        <v>24.79385100985203</v>
       </c>
       <c r="J81" s="2" t="n">
         <v>1.039332150141981</v>
@@ -4757,7 +4757,7 @@
         <v>-1</v>
       </c>
       <c r="N81" s="2" t="n">
-        <v>0.8985626879809949</v>
+        <v>0.8985626880840237</v>
       </c>
       <c r="O81" s="2" t="inlineStr">
         <is>
@@ -4792,10 +4792,10 @@
         <v>0</v>
       </c>
       <c r="H82" s="2" t="n">
-        <v>41.54752417994016</v>
+        <v>41.54752407679373</v>
       </c>
       <c r="I82" s="2" t="n">
-        <v>16.90533641229361</v>
+        <v>16.90533636579567</v>
       </c>
       <c r="J82" s="2" t="n">
         <v>1.066979638634609</v>
@@ -4810,7 +4810,7 @@
         <v>-1</v>
       </c>
       <c r="N82" s="2" t="n">
-        <v>-0.2449061345317567</v>
+        <v>-0.2449061343772147</v>
       </c>
       <c r="O82" s="2" t="inlineStr">
         <is>
@@ -4845,10 +4845,10 @@
         <v>0</v>
       </c>
       <c r="H83" s="2" t="n">
-        <v>56.71708472015602</v>
+        <v>56.71708471002968</v>
       </c>
       <c r="I83" s="2" t="n">
-        <v>19.73135405729172</v>
+        <v>19.73135399260932</v>
       </c>
       <c r="J83" s="2" t="n">
         <v>0.6181776551495262</v>
@@ -4863,7 +4863,7 @@
         <v>-1</v>
       </c>
       <c r="N83" s="2" t="n">
-        <v>-6.594915279924251</v>
+        <v>-6.594915279470897</v>
       </c>
       <c r="O83" s="2" t="inlineStr">
         <is>
@@ -4898,10 +4898,10 @@
         <v>0</v>
       </c>
       <c r="H84" s="2" t="n">
-        <v>40.03852034097489</v>
+        <v>40.03852032703208</v>
       </c>
       <c r="I84" s="2" t="n">
-        <v>23.52983322374143</v>
+        <v>23.52983315747493</v>
       </c>
       <c r="J84" s="2" t="n">
         <v>0.6791657215905617</v>
@@ -4916,7 +4916,7 @@
         <v>-1</v>
       </c>
       <c r="N84" s="2" t="n">
-        <v>-1.691758834387493</v>
+        <v>-1.691758834490517</v>
       </c>
       <c r="O84" s="2" t="inlineStr">
         <is>
@@ -4937,7 +4937,7 @@
         <v/>
       </c>
       <c r="D85" s="2" t="n">
-        <v>508.078195275117</v>
+        <v>508.078195275139</v>
       </c>
       <c r="E85" s="2" t="n">
         <v>19.45</v>
@@ -4951,10 +4951,10 @@
         <v>0</v>
       </c>
       <c r="H85" s="2" t="n">
-        <v>54.3392014804355</v>
+        <v>54.33920140859499</v>
       </c>
       <c r="I85" s="2" t="n">
-        <v>21.57790086597567</v>
+        <v>21.57790086313708</v>
       </c>
       <c r="J85" s="2" t="n">
         <v>1.076870314244696</v>
@@ -4969,7 +4969,7 @@
         <v>-1</v>
       </c>
       <c r="N85" s="2" t="n">
-        <v>0.0071054152076421</v>
+        <v>0.0071054151767313</v>
       </c>
       <c r="O85" s="2" t="inlineStr">
         <is>
@@ -4990,7 +4990,7 @@
         <v/>
       </c>
       <c r="D86" s="2" t="n">
-        <v>494.8256968700635</v>
+        <v>494.8256968700659</v>
       </c>
       <c r="E86" s="2" t="n">
         <v>30.3</v>
@@ -5004,10 +5004,10 @@
         <v>0</v>
       </c>
       <c r="H86" s="2" t="n">
-        <v>51.13007408082667</v>
+        <v>51.13007392037413</v>
       </c>
       <c r="I86" s="2" t="n">
-        <v>28.1614193460271</v>
+        <v>28.16141929293398</v>
       </c>
       <c r="J86" s="2" t="n">
         <v>0.910682592219504</v>
@@ -5022,7 +5022,7 @@
         <v>-1</v>
       </c>
       <c r="N86" s="2" t="n">
-        <v>0.0027794375345141</v>
+        <v>0.0027794378435997</v>
       </c>
       <c r="O86" s="2" t="inlineStr">
         <is>
@@ -5057,10 +5057,10 @@
         <v>0</v>
       </c>
       <c r="H87" s="2" t="n">
-        <v>46.27989437316214</v>
+        <v>46.27989439009651</v>
       </c>
       <c r="I87" s="2" t="n">
-        <v>21.12118768603549</v>
+        <v>21.12118781112725</v>
       </c>
       <c r="J87" s="2" t="n">
         <v>0.5566707479236955</v>
@@ -5075,7 +5075,7 @@
         <v>-1</v>
       </c>
       <c r="N87" s="2" t="n">
-        <v>-0.7519994212421002</v>
+        <v>-0.7519994207475615</v>
       </c>
       <c r="O87" s="2" t="inlineStr">
         <is>
@@ -5110,10 +5110,10 @@
         <v>0</v>
       </c>
       <c r="H88" s="2" t="n">
-        <v>48.64108792372458</v>
+        <v>48.64108789669236</v>
       </c>
       <c r="I88" s="2" t="n">
-        <v>24.41547653635058</v>
+        <v>24.41547647847264</v>
       </c>
       <c r="J88" s="2" t="n">
         <v>0.4328734432670099</v>
@@ -5128,7 +5128,7 @@
         <v>-1</v>
       </c>
       <c r="N88" s="2" t="n">
-        <v>-0.2370620691586248</v>
+        <v>-0.2370620690762003</v>
       </c>
       <c r="O88" s="2" t="inlineStr">
         <is>
@@ -5163,10 +5163,10 @@
         <v>0</v>
       </c>
       <c r="H89" s="2" t="n">
-        <v>49.40678641622087</v>
+        <v>49.4067863708441</v>
       </c>
       <c r="I89" s="2" t="n">
-        <v>13.5440760769691</v>
+        <v>13.54407603266381</v>
       </c>
       <c r="J89" s="2" t="n">
         <v>0.8210749930922494</v>
@@ -5181,7 +5181,7 @@
         <v>-1</v>
       </c>
       <c r="N89" s="2" t="n">
-        <v>0.0533812637746787</v>
+        <v>0.0533812638880123</v>
       </c>
       <c r="O89" s="2" t="inlineStr">
         <is>
@@ -5202,7 +5202,7 @@
         <v/>
       </c>
       <c r="D90" s="2" t="n">
-        <v>486.1273082555173</v>
+        <v>486.1273082555171</v>
       </c>
       <c r="E90" s="2" t="n">
         <v>89.2</v>
@@ -5216,10 +5216,10 @@
         <v>0</v>
       </c>
       <c r="H90" s="2" t="n">
-        <v>46.15825862098276</v>
+        <v>46.1582585321494</v>
       </c>
       <c r="I90" s="2" t="n">
-        <v>18.03236745905154</v>
+        <v>18.032367434237</v>
       </c>
       <c r="J90" s="2" t="n">
         <v>0.3470467695915137</v>
@@ -5234,7 +5234,7 @@
         <v>-1</v>
       </c>
       <c r="N90" s="2" t="n">
-        <v>-1.235308242490957</v>
+        <v>-1.235308241419458</v>
       </c>
       <c r="O90" s="2" t="inlineStr">
         <is>
@@ -5269,7 +5269,7 @@
         <v>0</v>
       </c>
       <c r="H91" s="2" t="n">
-        <v>51.81932553005295</v>
+        <v>51.81932551388644</v>
       </c>
       <c r="I91" s="2" t="n">
         <v>21.83650373460087</v>
@@ -5287,7 +5287,7 @@
         <v>-1</v>
       </c>
       <c r="N91" s="2" t="n">
-        <v>-0.1377733709200554</v>
+        <v>-0.1377733708994453</v>
       </c>
       <c r="O91" s="2" t="inlineStr">
         <is>
@@ -5322,10 +5322,10 @@
         <v>0</v>
       </c>
       <c r="H92" s="2" t="n">
-        <v>45.31986142022422</v>
+        <v>45.31986140707502</v>
       </c>
       <c r="I92" s="2" t="n">
-        <v>22.29854991528113</v>
+        <v>22.29854988780701</v>
       </c>
       <c r="J92" s="2" t="n">
         <v>1.130264392557432</v>
@@ -5340,7 +5340,7 @@
         <v>-1</v>
       </c>
       <c r="N92" s="2" t="n">
-        <v>-4.238519844953173</v>
+        <v>-4.238519844644085</v>
       </c>
       <c r="O92" s="2" t="inlineStr">
         <is>
@@ -5375,10 +5375,10 @@
         <v>0</v>
       </c>
       <c r="H93" s="2" t="n">
-        <v>51.49767503005823</v>
+        <v>51.49767502238681</v>
       </c>
       <c r="I93" s="2" t="n">
-        <v>17.77835321750136</v>
+        <v>17.77835323251475</v>
       </c>
       <c r="J93" s="2" t="n">
         <v>0.4375855515266134</v>
@@ -5393,7 +5393,7 @@
         <v>-1</v>
       </c>
       <c r="N93" s="2" t="n">
-        <v>-0.5194588379664729</v>
+        <v>-0.5194588379561752</v>
       </c>
       <c r="O93" s="2" t="inlineStr">
         <is>
@@ -5428,10 +5428,10 @@
         <v>0</v>
       </c>
       <c r="H94" s="2" t="n">
-        <v>54.97630133550902</v>
+        <v>54.97630131951047</v>
       </c>
       <c r="I94" s="2" t="n">
-        <v>15.92667408485208</v>
+        <v>15.92667403683286</v>
       </c>
       <c r="J94" s="2" t="n">
         <v>0.7947251712322165</v>
@@ -5446,7 +5446,7 @@
         <v>-1</v>
       </c>
       <c r="N94" s="2" t="n">
-        <v>1.774365781710001</v>
+        <v>1.774365782122097</v>
       </c>
       <c r="O94" s="2" t="inlineStr">
         <is>
@@ -5467,7 +5467,7 @@
         <v/>
       </c>
       <c r="D95" s="2" t="n">
-        <v>460.9256516745393</v>
+        <v>460.9256516745394</v>
       </c>
       <c r="E95" s="2" t="n">
         <v>45.4</v>
@@ -5481,10 +5481,10 @@
         <v>0</v>
       </c>
       <c r="H95" s="2" t="n">
-        <v>47.68063932692799</v>
+        <v>47.680639308727</v>
       </c>
       <c r="I95" s="2" t="n">
-        <v>16.79105254610824</v>
+        <v>16.7910525177039</v>
       </c>
       <c r="J95" s="2" t="n">
         <v>0.2815390684113325</v>
@@ -5499,7 +5499,7 @@
         <v>-1</v>
       </c>
       <c r="N95" s="2" t="n">
-        <v>-0.2967740865876499</v>
+        <v>-0.2967740869379448</v>
       </c>
       <c r="O95" s="2" t="inlineStr">
         <is>
@@ -5534,10 +5534,10 @@
         <v>0</v>
       </c>
       <c r="H96" s="2" t="n">
-        <v>58.66082964183292</v>
+        <v>58.66082931965958</v>
       </c>
       <c r="I96" s="2" t="n">
-        <v>27.37963574479512</v>
+        <v>27.37963576112145</v>
       </c>
       <c r="J96" s="2" t="n">
         <v>0.6870802112402674</v>
@@ -5552,7 +5552,7 @@
         <v>-1</v>
       </c>
       <c r="N96" s="2" t="n">
-        <v>0.0383160401583699</v>
+        <v>0.0383160401789763</v>
       </c>
       <c r="O96" s="2" t="inlineStr">
         <is>
@@ -5573,7 +5573,7 @@
         <v/>
       </c>
       <c r="D97" s="2" t="n">
-        <v>452.051348521343</v>
+        <v>452.0513485213419</v>
       </c>
       <c r="E97" s="2" t="n">
         <v>43</v>
@@ -5587,10 +5587,10 @@
         <v>0</v>
       </c>
       <c r="H97" s="2" t="n">
-        <v>49.14142798590154</v>
+        <v>49.14142792163661</v>
       </c>
       <c r="I97" s="2" t="n">
-        <v>10.62189796747961</v>
+        <v>10.62189783920204</v>
       </c>
       <c r="J97" s="2" t="n">
         <v>0.4476298264446404</v>
@@ -5605,7 +5605,7 @@
         <v>-1</v>
       </c>
       <c r="N97" s="2" t="n">
-        <v>-0.2784912587177294</v>
+        <v>-0.2784912583983436</v>
       </c>
       <c r="O97" s="2" t="inlineStr">
         <is>
@@ -5640,10 +5640,10 @@
         <v>0</v>
       </c>
       <c r="H98" s="2" t="n">
-        <v>47.66339629693615</v>
+        <v>47.66339628436477</v>
       </c>
       <c r="I98" s="2" t="n">
-        <v>14.39523286273986</v>
+        <v>14.39523284936156</v>
       </c>
       <c r="J98" s="2" t="n">
         <v>1.38884627264462</v>
@@ -5658,7 +5658,7 @@
         <v>-1</v>
       </c>
       <c r="N98" s="2" t="n">
-        <v>-2.702144510589301</v>
+        <v>-2.702144509971095</v>
       </c>
       <c r="O98" s="2" t="inlineStr">
         <is>
@@ -5696,7 +5696,7 @@
         <v>48.27942613318452</v>
       </c>
       <c r="I99" s="2" t="n">
-        <v>26.36888225736968</v>
+        <v>26.36888221413547</v>
       </c>
       <c r="J99" s="2" t="n">
         <v>0.4662280143248132</v>
@@ -5711,7 +5711,7 @@
         <v>-1</v>
       </c>
       <c r="N99" s="2" t="n">
-        <v>-0.1660859253761011</v>
+        <v>-0.1660859253554954</v>
       </c>
       <c r="O99" s="2" t="inlineStr">
         <is>
@@ -5746,10 +5746,10 @@
         <v>0</v>
       </c>
       <c r="H100" s="2" t="n">
-        <v>56.7887863077765</v>
+        <v>56.78878622321243</v>
       </c>
       <c r="I100" s="2" t="n">
-        <v>19.55214851575866</v>
+        <v>19.55214849022409</v>
       </c>
       <c r="J100" s="2" t="n">
         <v>1.134935991753811</v>
@@ -5764,7 +5764,7 @@
         <v>-1</v>
       </c>
       <c r="N100" s="2" t="n">
-        <v>0.1688809441414356</v>
+        <v>0.1688809446977892</v>
       </c>
       <c r="O100" s="2" t="inlineStr">
         <is>
@@ -5799,10 +5799,10 @@
         <v>0</v>
       </c>
       <c r="H101" s="2" t="n">
-        <v>53.88486499596873</v>
+        <v>53.88486498393376</v>
       </c>
       <c r="I101" s="2" t="n">
-        <v>28.44029323470052</v>
+        <v>28.44029326522423</v>
       </c>
       <c r="J101" s="2" t="n">
         <v>0.8762021481385343</v>
@@ -5817,7 +5817,7 @@
         <v>-1</v>
       </c>
       <c r="N101" s="2" t="n">
-        <v>-0.1226050620721904</v>
+        <v>-0.1226050621031008</v>
       </c>
       <c r="O101" s="2" t="inlineStr">
         <is>
@@ -5852,10 +5852,10 @@
         <v>0</v>
       </c>
       <c r="H102" s="2" t="n">
-        <v>48.47810670559073</v>
+        <v>48.47810660558223</v>
       </c>
       <c r="I102" s="2" t="n">
-        <v>23.16180222455658</v>
+        <v>23.16180237896469</v>
       </c>
       <c r="J102" s="2" t="n">
         <v>1.242767711464073</v>
@@ -5870,7 +5870,7 @@
         <v>-1</v>
       </c>
       <c r="N102" s="2" t="n">
-        <v>-0.07728164015874189</v>
+        <v>-0.07728163983935531</v>
       </c>
       <c r="O102" s="2" t="inlineStr">
         <is>
@@ -5905,10 +5905,10 @@
         <v>0</v>
       </c>
       <c r="H103" s="2" t="n">
-        <v>54.37556473156123</v>
+        <v>54.37556453760648</v>
       </c>
       <c r="I103" s="2" t="n">
-        <v>12.02787975920139</v>
+        <v>12.02787980604684</v>
       </c>
       <c r="J103" s="2" t="n">
         <v>0.5712116984751362</v>
@@ -5923,7 +5923,7 @@
         <v>-1</v>
       </c>
       <c r="N103" s="2" t="n">
-        <v>-0.013824367228062</v>
+        <v>-0.0138243670838256</v>
       </c>
       <c r="O103" s="2" t="inlineStr">
         <is>
@@ -5958,10 +5958,10 @@
         <v>0</v>
       </c>
       <c r="H104" s="2" t="n">
-        <v>40.66149967383327</v>
+        <v>40.66149962010821</v>
       </c>
       <c r="I104" s="2" t="n">
-        <v>8.592170506995599</v>
+        <v>8.592170439634469</v>
       </c>
       <c r="J104" s="2" t="n">
         <v>1.014115745617696</v>
@@ -5976,7 +5976,7 @@
         <v>-1</v>
       </c>
       <c r="N104" s="2" t="n">
-        <v>-0.08474586959800599</v>
+        <v>-0.0847458695629764</v>
       </c>
       <c r="O104" s="2" t="inlineStr">
         <is>
@@ -6011,10 +6011,10 @@
         <v>0</v>
       </c>
       <c r="H105" s="2" t="n">
-        <v>51.75523107233126</v>
+        <v>51.75523106703744</v>
       </c>
       <c r="I105" s="2" t="n">
-        <v>8.224408669297645</v>
+        <v>8.22440873207524</v>
       </c>
       <c r="J105" s="2" t="n">
         <v>1.196465971737404</v>
@@ -6029,7 +6029,7 @@
         <v>-1</v>
       </c>
       <c r="N105" s="2" t="n">
-        <v>1.098267625417927</v>
+        <v>1.098267625747622</v>
       </c>
       <c r="O105" s="2" t="inlineStr">
         <is>
@@ -6064,10 +6064,10 @@
         <v>0</v>
       </c>
       <c r="H106" s="2" t="n">
-        <v>55.03181164209622</v>
+        <v>55.03181149701678</v>
       </c>
       <c r="I106" s="2" t="n">
-        <v>13.65521451596129</v>
+        <v>13.65521456974597</v>
       </c>
       <c r="J106" s="2" t="n">
         <v>0.7550570032758982</v>
@@ -6082,7 +6082,7 @@
         <v>-1</v>
       </c>
       <c r="N106" s="2" t="n">
-        <v>-0.0326150513586045</v>
+        <v>-0.0326150510289022</v>
       </c>
       <c r="O106" s="2" t="inlineStr">
         <is>
@@ -6117,10 +6117,10 @@
         <v>0</v>
       </c>
       <c r="H107" s="2" t="n">
-        <v>48.75601391372039</v>
+        <v>48.75601385435604</v>
       </c>
       <c r="I107" s="2" t="n">
-        <v>6.396115724418991</v>
+        <v>6.396115708653912</v>
       </c>
       <c r="J107" s="2" t="n">
         <v>1.533229889574869</v>
@@ -6135,7 +6135,7 @@
         <v>-1</v>
       </c>
       <c r="N107" s="2" t="n">
-        <v>0.3039489590719899</v>
+        <v>0.303948959504706</v>
       </c>
       <c r="O107" s="2" t="inlineStr">
         <is>
@@ -6170,10 +6170,10 @@
         <v>0</v>
       </c>
       <c r="H108" s="2" t="n">
-        <v>47.56696961749569</v>
+        <v>47.56696952276996</v>
       </c>
       <c r="I108" s="2" t="n">
-        <v>20.59056001054423</v>
+        <v>20.59055986602495</v>
       </c>
       <c r="J108" s="2" t="n">
         <v>0.5266392464178679</v>
@@ -6188,7 +6188,7 @@
         <v>-1</v>
       </c>
       <c r="N108" s="2" t="n">
-        <v>-0.4475760155641639</v>
+        <v>-0.4475760148017489</v>
       </c>
       <c r="O108" s="2" t="inlineStr">
         <is>
@@ -6209,7 +6209,7 @@
         <v/>
       </c>
       <c r="D109" s="2" t="n">
-        <v>389.6831980420388</v>
+        <v>389.6831980420391</v>
       </c>
       <c r="E109" s="2" t="n">
         <v>400</v>
@@ -6223,10 +6223,10 @@
         <v>0</v>
       </c>
       <c r="H109" s="2" t="n">
-        <v>49.62739523050602</v>
+        <v>49.62739521754296</v>
       </c>
       <c r="I109" s="2" t="n">
-        <v>15.62496926515464</v>
+        <v>15.62496922785751</v>
       </c>
       <c r="J109" s="2" t="n">
         <v>0.5912670512640484</v>
@@ -6241,7 +6241,7 @@
         <v>-1</v>
       </c>
       <c r="N109" s="2" t="n">
-        <v>0.2226670986352408</v>
+        <v>0.2226670989442993</v>
       </c>
       <c r="O109" s="2" t="inlineStr">
         <is>
@@ -6276,10 +6276,10 @@
         <v>0</v>
       </c>
       <c r="H110" s="2" t="n">
-        <v>47.29329688470292</v>
+        <v>47.29329447025658</v>
       </c>
       <c r="I110" s="2" t="n">
-        <v>17.33416056846341</v>
+        <v>17.3341612705978</v>
       </c>
       <c r="J110" s="2" t="n">
         <v>0.88165361832567</v>
@@ -6294,7 +6294,7 @@
         <v>-1</v>
       </c>
       <c r="N110" s="2" t="n">
-        <v>0.1405135771571359</v>
+        <v>0.1405135842661384</v>
       </c>
       <c r="O110" s="2" t="inlineStr">
         <is>
@@ -6315,7 +6315,7 @@
         <v/>
       </c>
       <c r="D111" s="2" t="n">
-        <v>386.9070414143378</v>
+        <v>386.9070414143379</v>
       </c>
       <c r="E111" s="2" t="n">
         <v>38.25</v>
@@ -6329,10 +6329,10 @@
         <v>0</v>
       </c>
       <c r="H111" s="2" t="n">
-        <v>48.09688569743324</v>
+        <v>48.09688541712121</v>
       </c>
       <c r="I111" s="2" t="n">
-        <v>11.62843014328742</v>
+        <v>11.62843009957894</v>
       </c>
       <c r="J111" s="2" t="n">
         <v>0.5738289596749503</v>
@@ -6347,7 +6347,7 @@
         <v>-1</v>
       </c>
       <c r="N111" s="2" t="n">
-        <v>0.0598560250206913</v>
+        <v>0.0598560253091704</v>
       </c>
       <c r="O111" s="2" t="inlineStr">
         <is>
@@ -6382,10 +6382,10 @@
         <v>0</v>
       </c>
       <c r="H112" s="2" t="n">
-        <v>53.23811751704128</v>
+        <v>53.23811749922012</v>
       </c>
       <c r="I112" s="2" t="n">
-        <v>21.18102860665202</v>
+        <v>21.18102854078862</v>
       </c>
       <c r="J112" s="2" t="n">
         <v>0.4436337318091758</v>
@@ -6400,7 +6400,7 @@
         <v>-1</v>
       </c>
       <c r="N112" s="2" t="n">
-        <v>0.0177681413078498</v>
+        <v>0.017768141390272</v>
       </c>
       <c r="O112" s="2" t="inlineStr">
         <is>
@@ -6435,10 +6435,10 @@
         <v>0</v>
       </c>
       <c r="H113" s="2" t="n">
-        <v>43.96097942134539</v>
+        <v>43.96097905493917</v>
       </c>
       <c r="I113" s="2" t="n">
-        <v>20.69618242313008</v>
+        <v>20.6961822286978</v>
       </c>
       <c r="J113" s="2" t="n">
         <v>0.4498870432542391</v>
@@ -6453,7 +6453,7 @@
         <v>-1</v>
       </c>
       <c r="N113" s="2" t="n">
-        <v>-3.307064781315299</v>
+        <v>-3.307064774721437</v>
       </c>
       <c r="O113" s="2" t="inlineStr">
         <is>
@@ -6488,10 +6488,10 @@
         <v>0</v>
       </c>
       <c r="H114" s="2" t="n">
-        <v>53.33773454654397</v>
+        <v>53.3377345209229</v>
       </c>
       <c r="I114" s="2" t="n">
-        <v>30.42790734967763</v>
+        <v>30.42790732852828</v>
       </c>
       <c r="J114" s="2" t="n">
         <v>0.5718590558221669</v>
@@ -6506,7 +6506,7 @@
         <v>-1</v>
       </c>
       <c r="N114" s="2" t="n">
-        <v>-0.4309912469565755</v>
+        <v>-0.430991246822637</v>
       </c>
       <c r="O114" s="2" t="inlineStr">
         <is>
@@ -6541,10 +6541,10 @@
         <v>0</v>
       </c>
       <c r="H115" s="2" t="n">
-        <v>47.49488756359949</v>
+        <v>47.49488755859812</v>
       </c>
       <c r="I115" s="2" t="n">
-        <v>19.1833113409706</v>
+        <v>19.18331134073462</v>
       </c>
       <c r="J115" s="2" t="n">
         <v>0.5750011354340985</v>
@@ -6559,7 +6559,7 @@
         <v>-1</v>
       </c>
       <c r="N115" s="2" t="n">
-        <v>-11.79238581361959</v>
+        <v>-11.7923858121772</v>
       </c>
       <c r="O115" s="2" t="inlineStr">
         <is>
@@ -6580,7 +6580,7 @@
         <v/>
       </c>
       <c r="D116" s="2" t="n">
-        <v>364.014810902731</v>
+        <v>364.0148109027309</v>
       </c>
       <c r="E116" s="2" t="n">
         <v>73.90000000000001</v>
@@ -6594,10 +6594,10 @@
         <v>0</v>
       </c>
       <c r="H116" s="2" t="n">
-        <v>51.47576613003636</v>
+        <v>51.47576589604767</v>
       </c>
       <c r="I116" s="2" t="n">
-        <v>22.73009331477247</v>
+        <v>22.7300938109553</v>
       </c>
       <c r="J116" s="2" t="n">
         <v>0.4967510372944574</v>
@@ -6612,7 +6612,7 @@
         <v>-1</v>
       </c>
       <c r="N116" s="2" t="n">
-        <v>0.338095117951986</v>
+        <v>0.3380951198065183</v>
       </c>
       <c r="O116" s="2" t="inlineStr">
         <is>
@@ -6647,10 +6647,10 @@
         <v>0</v>
       </c>
       <c r="H117" s="2" t="n">
-        <v>44.81393938021723</v>
+        <v>44.81393935922982</v>
       </c>
       <c r="I117" s="2" t="n">
-        <v>13.37207794378714</v>
+        <v>13.37207797960278</v>
       </c>
       <c r="J117" s="2" t="n">
         <v>0.9969259656539706</v>
@@ -6665,7 +6665,7 @@
         <v>-1</v>
       </c>
       <c r="N117" s="2" t="n">
-        <v>0.3256731813559499</v>
+        <v>0.3256731813353439</v>
       </c>
       <c r="O117" s="2" t="inlineStr">
         <is>
@@ -6700,10 +6700,10 @@
         <v>0</v>
       </c>
       <c r="H118" s="2" t="n">
-        <v>52.68454888081687</v>
+        <v>52.68454888622483</v>
       </c>
       <c r="I118" s="2" t="n">
-        <v>11.99270689096185</v>
+        <v>11.99270686119043</v>
       </c>
       <c r="J118" s="2" t="n">
         <v>0.2797336035404054</v>
@@ -6718,7 +6718,7 @@
         <v>-1</v>
       </c>
       <c r="N118" s="2" t="n">
-        <v>-0.1131611799906293</v>
+        <v>-0.1131611800112355</v>
       </c>
       <c r="O118" s="2" t="inlineStr">
         <is>
@@ -6753,10 +6753,10 @@
         <v>0</v>
       </c>
       <c r="H119" s="2" t="n">
-        <v>51.61779906907893</v>
+        <v>51.6177990289138</v>
       </c>
       <c r="I119" s="2" t="n">
-        <v>27.10866584102615</v>
+        <v>27.10866597930893</v>
       </c>
       <c r="J119" s="2" t="n">
         <v>0.8745899314395879</v>
@@ -6771,7 +6771,7 @@
         <v>-1</v>
       </c>
       <c r="N119" s="2" t="n">
-        <v>0.0801505075947682</v>
+        <v>0.08015050764628411</v>
       </c>
       <c r="O119" s="2" t="inlineStr">
         <is>
@@ -6792,7 +6792,7 @@
         <v/>
       </c>
       <c r="D120" s="2" t="n">
-        <v>359.1505040153397</v>
+        <v>359.1505040153396</v>
       </c>
       <c r="E120" s="2" t="n">
         <v>51.3</v>
@@ -6806,10 +6806,10 @@
         <v>0</v>
       </c>
       <c r="H120" s="2" t="n">
-        <v>50.17899869290245</v>
+        <v>50.17899859823535</v>
       </c>
       <c r="I120" s="2" t="n">
-        <v>16.02524226863864</v>
+        <v>16.02524229372656</v>
       </c>
       <c r="J120" s="2" t="n">
         <v>0.7303552295959654</v>
@@ -6824,7 +6824,7 @@
         <v>-1</v>
       </c>
       <c r="N120" s="2" t="n">
-        <v>-0.0320390672756403</v>
+        <v>-0.0320390673992773</v>
       </c>
       <c r="O120" s="2" t="inlineStr">
         <is>
@@ -6859,10 +6859,10 @@
         <v>0</v>
       </c>
       <c r="H121" s="2" t="n">
-        <v>44.06723989343447</v>
+        <v>44.06723987652316</v>
       </c>
       <c r="I121" s="2" t="n">
-        <v>20.02589041823146</v>
+        <v>20.02589047081349</v>
       </c>
       <c r="J121" s="2" t="n">
         <v>0.5515148495743272</v>
@@ -6877,7 +6877,7 @@
         <v>-1</v>
       </c>
       <c r="N121" s="2" t="n">
-        <v>-0.5244377284924928</v>
+        <v>-0.524437728379163</v>
       </c>
       <c r="O121" s="2" t="inlineStr">
         <is>
@@ -6898,7 +6898,7 @@
         <v/>
       </c>
       <c r="D122" s="2" t="n">
-        <v>347.0956456458615</v>
+        <v>347.0956456458607</v>
       </c>
       <c r="E122" s="2" t="n">
         <v>49.85</v>
@@ -6912,10 +6912,10 @@
         <v>0</v>
       </c>
       <c r="H122" s="2" t="n">
-        <v>43.12857165293004</v>
+        <v>43.12857142901406</v>
       </c>
       <c r="I122" s="2" t="n">
-        <v>26.97953154576333</v>
+        <v>26.97953168873717</v>
       </c>
       <c r="J122" s="2" t="n">
         <v>0.7196850882026196</v>
@@ -6930,7 +6930,7 @@
         <v>-1</v>
       </c>
       <c r="N122" s="2" t="n">
-        <v>0.1528612130714157</v>
+        <v>0.1528612134423235</v>
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
@@ -6965,10 +6965,10 @@
         <v>0</v>
       </c>
       <c r="H123" s="2" t="n">
-        <v>51.70967044690357</v>
+        <v>51.70967022629937</v>
       </c>
       <c r="I123" s="2" t="n">
-        <v>12.56036457875766</v>
+        <v>12.56036453140282</v>
       </c>
       <c r="J123" s="2" t="n">
         <v>3.437218445409124</v>
@@ -6983,7 +6983,7 @@
         <v>-1</v>
       </c>
       <c r="N123" s="2" t="n">
-        <v>0.0179757027670349</v>
+        <v>0.0179757029318823</v>
       </c>
       <c r="O123" s="2" t="inlineStr">
         <is>
@@ -7018,10 +7018,10 @@
         <v>0</v>
       </c>
       <c r="H124" s="2" t="n">
-        <v>42.45085875996646</v>
+        <v>42.45085866789984</v>
       </c>
       <c r="I124" s="2" t="n">
-        <v>21.22152970457825</v>
+        <v>21.22152962280965</v>
       </c>
       <c r="J124" s="2" t="n">
         <v>0.5636686818405192</v>
@@ -7036,7 +7036,7 @@
         <v>-1</v>
       </c>
       <c r="N124" s="2" t="n">
-        <v>-1.365318457586716</v>
+        <v>-1.365318456844905</v>
       </c>
       <c r="O124" s="2" t="inlineStr">
         <is>
@@ -7071,10 +7071,10 @@
         <v>0</v>
       </c>
       <c r="H125" s="2" t="n">
-        <v>46.88714134446358</v>
+        <v>46.88714131998224</v>
       </c>
       <c r="I125" s="2" t="n">
-        <v>14.3322778979312</v>
+        <v>14.33227780137412</v>
       </c>
       <c r="J125" s="2" t="n">
         <v>0.6665159657628114</v>
@@ -7089,7 +7089,7 @@
         <v>-1</v>
       </c>
       <c r="N125" s="2" t="n">
-        <v>-1.414236434373574</v>
+        <v>-1.414236434198411</v>
       </c>
       <c r="O125" s="2" t="inlineStr">
         <is>
@@ -7124,10 +7124,10 @@
         <v>0</v>
       </c>
       <c r="H126" s="2" t="n">
-        <v>42.55684782886682</v>
+        <v>42.55684778275923</v>
       </c>
       <c r="I126" s="2" t="n">
-        <v>29.6467169186758</v>
+        <v>29.64671692385884</v>
       </c>
       <c r="J126" s="2" t="n">
         <v>0.8150938087815007</v>
@@ -7142,7 +7142,7 @@
         <v>-1</v>
       </c>
       <c r="N126" s="2" t="n">
-        <v>-2.210377044515215</v>
+        <v>-2.21037704420614</v>
       </c>
       <c r="O126" s="2" t="inlineStr">
         <is>
@@ -7177,10 +7177,10 @@
         <v>0</v>
       </c>
       <c r="H127" s="2" t="n">
-        <v>50.64963752852788</v>
+        <v>50.64963748827503</v>
       </c>
       <c r="I127" s="2" t="n">
-        <v>12.52516739925081</v>
+        <v>12.52516735041737</v>
       </c>
       <c r="J127" s="2" t="n">
         <v>0.4294168940808016</v>
@@ -7195,7 +7195,7 @@
         <v>-1</v>
       </c>
       <c r="N127" s="2" t="n">
-        <v>-0.0681026311802598</v>
+        <v>-0.0681026311390478</v>
       </c>
       <c r="O127" s="2" t="inlineStr">
         <is>
@@ -7216,7 +7216,7 @@
         <v/>
       </c>
       <c r="D128" s="2" t="n">
-        <v>301.686907658094</v>
+        <v>301.6869076580939</v>
       </c>
       <c r="E128" s="2" t="n">
         <v>24.25</v>
@@ -7230,10 +7230,10 @@
         <v>0</v>
       </c>
       <c r="H128" s="2" t="n">
-        <v>52.21272220233155</v>
+        <v>52.21272222131246</v>
       </c>
       <c r="I128" s="2" t="n">
-        <v>17.77136394383433</v>
+        <v>17.77136394820672</v>
       </c>
       <c r="J128" s="2" t="n">
         <v>0.5801747959548423</v>
@@ -7248,7 +7248,7 @@
         <v>-1</v>
       </c>
       <c r="N128" s="2" t="n">
-        <v>0.08425600109714319</v>
+        <v>0.0842560011280509</v>
       </c>
       <c r="O128" s="2" t="inlineStr">
         <is>
@@ -7283,10 +7283,10 @@
         <v>0</v>
       </c>
       <c r="H129" s="2" t="n">
-        <v>44.88846684404455</v>
+        <v>44.88846668924081</v>
       </c>
       <c r="I129" s="2" t="n">
-        <v>15.24971792465494</v>
+        <v>15.24971800919818</v>
       </c>
       <c r="J129" s="2" t="n">
         <v>0.904028017143364</v>
@@ -7301,7 +7301,7 @@
         <v>-1</v>
       </c>
       <c r="N129" s="2" t="n">
-        <v>-0.6690023295442539</v>
+        <v>-0.6690023288230524</v>
       </c>
       <c r="O129" s="2" t="inlineStr">
         <is>
@@ -7336,10 +7336,10 @@
         <v>0</v>
       </c>
       <c r="H130" s="2" t="n">
-        <v>51.58334717630207</v>
+        <v>51.5833471642728</v>
       </c>
       <c r="I130" s="2" t="n">
-        <v>19.51138362079003</v>
+        <v>19.51138352338874</v>
       </c>
       <c r="J130" s="2" t="n">
         <v>0.6104345616794977</v>
@@ -7354,7 +7354,7 @@
         <v>-1</v>
       </c>
       <c r="N130" s="2" t="n">
-        <v>0.0215310586016959</v>
+        <v>0.0215310586078768</v>
       </c>
       <c r="O130" s="2" t="inlineStr">
         <is>
@@ -7389,10 +7389,10 @@
         <v>0</v>
       </c>
       <c r="H131" s="2" t="n">
-        <v>49.17583809032821</v>
+        <v>49.17583803143717</v>
       </c>
       <c r="I131" s="2" t="n">
-        <v>12.21962031350802</v>
+        <v>12.21962035446313</v>
       </c>
       <c r="J131" s="2" t="n">
         <v>0.6907490283679751</v>
@@ -7407,7 +7407,7 @@
         <v>-1</v>
       </c>
       <c r="N131" s="2" t="n">
-        <v>-0.0268249591886586</v>
+        <v>-0.0268249591371415</v>
       </c>
       <c r="O131" s="2" t="inlineStr">
         <is>
@@ -7442,10 +7442,10 @@
         <v>0</v>
       </c>
       <c r="H132" s="2" t="n">
-        <v>39.19192491365048</v>
+        <v>39.1919247293265</v>
       </c>
       <c r="I132" s="2" t="n">
-        <v>12.87151849464274</v>
+        <v>12.87151845686592</v>
       </c>
       <c r="J132" s="2" t="n">
         <v>1.236607936165212</v>
@@ -7460,7 +7460,7 @@
         <v>-1</v>
       </c>
       <c r="N132" s="2" t="n">
-        <v>0.0195322229580362</v>
+        <v>0.0195322230095517</v>
       </c>
       <c r="O132" s="2" t="inlineStr">
         <is>
@@ -7495,10 +7495,10 @@
         <v>0</v>
       </c>
       <c r="H133" s="2" t="n">
-        <v>46.07197462005743</v>
+        <v>46.07197458878338</v>
       </c>
       <c r="I133" s="2" t="n">
-        <v>15.81563850118209</v>
+        <v>15.81563848342978</v>
       </c>
       <c r="J133" s="2" t="n">
         <v>1.053281424913042</v>
@@ -7513,7 +7513,7 @@
         <v>-1</v>
       </c>
       <c r="N133" s="2" t="n">
-        <v>-5.732611041436428</v>
+        <v>-5.732611039066693</v>
       </c>
       <c r="O133" s="2" t="inlineStr">
         <is>
@@ -7548,10 +7548,10 @@
         <v>0</v>
       </c>
       <c r="H134" s="2" t="n">
-        <v>40.31343093046162</v>
+        <v>40.31343094210011</v>
       </c>
       <c r="I134" s="2" t="n">
-        <v>17.00893379852839</v>
+        <v>17.00893379372241</v>
       </c>
       <c r="J134" s="2" t="n">
         <v>0.8109664535504745</v>
@@ -7566,7 +7566,7 @@
         <v>-1</v>
       </c>
       <c r="N134" s="2" t="n">
-        <v>-0.7165802695551287</v>
+        <v>-0.7165802696787711</v>
       </c>
       <c r="O134" s="2" t="inlineStr">
         <is>
@@ -7601,10 +7601,10 @@
         <v>0</v>
       </c>
       <c r="H135" s="2" t="n">
-        <v>40.73434793626</v>
+        <v>40.73434767368921</v>
       </c>
       <c r="I135" s="2" t="n">
-        <v>19.73099319664384</v>
+        <v>19.73099325759885</v>
       </c>
       <c r="J135" s="2" t="n">
         <v>0.6414044209274942</v>
@@ -7619,7 +7619,7 @@
         <v>-1</v>
       </c>
       <c r="N135" s="2" t="n">
-        <v>-0.6353376160009399</v>
+        <v>-0.6353376154445735</v>
       </c>
       <c r="O135" s="2" t="inlineStr">
         <is>
@@ -7654,7 +7654,7 @@
         <v>0</v>
       </c>
       <c r="H136" s="2" t="n">
-        <v>48.02001813269803</v>
+        <v>48.02001807999454</v>
       </c>
       <c r="I136" s="2" t="n">
         <v>16.61432208656763</v>
@@ -7707,10 +7707,10 @@
         <v>0</v>
       </c>
       <c r="H137" s="2" t="n">
-        <v>41.27284530977168</v>
+        <v>41.27284528111535</v>
       </c>
       <c r="I137" s="2" t="n">
-        <v>19.32379224083203</v>
+        <v>19.32379220919432</v>
       </c>
       <c r="J137" s="2" t="n">
         <v>0.5862272562472456</v>
@@ -7725,7 +7725,7 @@
         <v>-1</v>
       </c>
       <c r="N137" s="2" t="n">
-        <v>-3.566129990865557</v>
+        <v>-3.566129990247358</v>
       </c>
       <c r="O137" s="2" t="inlineStr">
         <is>
@@ -7760,10 +7760,10 @@
         <v>0</v>
       </c>
       <c r="H138" s="2" t="n">
-        <v>50.1526260539116</v>
+        <v>50.15262603623229</v>
       </c>
       <c r="I138" s="2" t="n">
-        <v>15.10315179797463</v>
+        <v>15.10315171796386</v>
       </c>
       <c r="J138" s="2" t="n">
         <v>0.8830752369478884</v>
@@ -7778,7 +7778,7 @@
         <v>-1</v>
       </c>
       <c r="N138" s="2" t="n">
-        <v>-0.2424745829156014</v>
+        <v>-0.2424745827919651</v>
       </c>
       <c r="O138" s="2" t="inlineStr">
         <is>
@@ -7813,10 +7813,10 @@
         <v>0</v>
       </c>
       <c r="H139" s="2" t="n">
-        <v>40.54761268223947</v>
+        <v>40.54761266004356</v>
       </c>
       <c r="I139" s="2" t="n">
-        <v>16.31636435029005</v>
+        <v>16.31636427977497</v>
       </c>
       <c r="J139" s="2" t="n">
         <v>0.5395018911541646</v>
@@ -7831,7 +7831,7 @@
         <v>-1</v>
       </c>
       <c r="N139" s="2" t="n">
-        <v>-0.216929024071516</v>
+        <v>-0.2169290240200043</v>
       </c>
       <c r="O139" s="2" t="inlineStr">
         <is>
@@ -7866,10 +7866,10 @@
         <v>0</v>
       </c>
       <c r="H140" s="2" t="n">
-        <v>43.1718474469709</v>
+        <v>43.17184736734441</v>
       </c>
       <c r="I140" s="2" t="n">
-        <v>19.55809483363572</v>
+        <v>19.55809484982264</v>
       </c>
       <c r="J140" s="2" t="n">
         <v>0.2985557055919386</v>
@@ -7884,7 +7884,7 @@
         <v>-1</v>
       </c>
       <c r="N140" s="2" t="n">
-        <v>-0.7224622721104053</v>
+        <v>-0.7224622719455618</v>
       </c>
       <c r="O140" s="2" t="inlineStr">
         <is>
@@ -7919,10 +7919,10 @@
         <v>0</v>
       </c>
       <c r="H141" s="2" t="n">
-        <v>46.51827821381284</v>
+        <v>46.5182780757375</v>
       </c>
       <c r="I141" s="2" t="n">
-        <v>11.48072854052531</v>
+        <v>11.48072852345976</v>
       </c>
       <c r="J141" s="2" t="n">
         <v>1.097318016899507</v>
@@ -7937,7 +7937,7 @@
         <v>-1</v>
       </c>
       <c r="N141" s="2" t="n">
-        <v>-0.0796054804901697</v>
+        <v>-0.07960548046956401</v>
       </c>
       <c r="O141" s="2" t="inlineStr">
         <is>
@@ -7972,10 +7972,10 @@
         <v>0</v>
       </c>
       <c r="H142" s="2" t="n">
-        <v>46.280926412304</v>
+        <v>46.28092615010993</v>
       </c>
       <c r="I142" s="2" t="n">
-        <v>15.09903944476142</v>
+        <v>15.09903951282327</v>
       </c>
       <c r="J142" s="2" t="n">
         <v>0.7660894593516709</v>
@@ -7990,7 +7990,7 @@
         <v>-1</v>
       </c>
       <c r="N142" s="2" t="n">
-        <v>-0.0166532428682096</v>
+        <v>-0.016653242723969</v>
       </c>
       <c r="O142" s="2" t="inlineStr">
         <is>
@@ -8011,7 +8011,7 @@
         <v/>
       </c>
       <c r="D143" s="2" t="n">
-        <v>184.9150529736015</v>
+        <v>184.9150529736016</v>
       </c>
       <c r="E143" s="2" t="n">
         <v>91</v>
@@ -8025,10 +8025,10 @@
         <v>0</v>
       </c>
       <c r="H143" s="2" t="n">
-        <v>50.67044622806622</v>
+        <v>50.67044621796306</v>
       </c>
       <c r="I143" s="2" t="n">
-        <v>21.06809184656684</v>
+        <v>21.06809192004132</v>
       </c>
       <c r="J143" s="2" t="n">
         <v>0.3788868998363319</v>
@@ -8043,7 +8043,7 @@
         <v>-1</v>
       </c>
       <c r="N143" s="2" t="n">
-        <v>0.7725728579018789</v>
+        <v>0.7725728580255034</v>
       </c>
       <c r="O143" s="2" t="inlineStr">
         <is>
@@ -8078,10 +8078,10 @@
         <v>0</v>
       </c>
       <c r="H144" s="2" t="n">
-        <v>35.833025760789</v>
+        <v>35.83302559282981</v>
       </c>
       <c r="I144" s="2" t="n">
-        <v>19.63276166303504</v>
+        <v>19.63276182178926</v>
       </c>
       <c r="J144" s="2" t="n">
         <v>0.9315990009135168</v>
@@ -8096,7 +8096,7 @@
         <v>-1</v>
       </c>
       <c r="N144" s="2" t="n">
-        <v>-0.4182686766784845</v>
+        <v>-0.4182686765136442</v>
       </c>
       <c r="O144" s="2" t="inlineStr">
         <is>
@@ -8117,7 +8117,7 @@
         <v/>
       </c>
       <c r="D145" s="2" t="n">
-        <v>174.1900233652146</v>
+        <v>174.1900233652152</v>
       </c>
       <c r="E145" s="2" t="n">
         <v>571</v>
@@ -8131,10 +8131,10 @@
         <v>0</v>
       </c>
       <c r="H145" s="2" t="n">
-        <v>41.75951854413805</v>
+        <v>41.75951852704994</v>
       </c>
       <c r="I145" s="2" t="n">
-        <v>17.30912844369669</v>
+        <v>17.30912844532232</v>
       </c>
       <c r="J145" s="2" t="n">
         <v>1.383843661772505</v>
@@ -8149,7 +8149,7 @@
         <v>-1</v>
       </c>
       <c r="N145" s="2" t="n">
-        <v>-7.729366551295456</v>
+        <v>-7.729366550368262</v>
       </c>
       <c r="O145" s="2" t="inlineStr">
         <is>
@@ -8184,10 +8184,10 @@
         <v>0</v>
       </c>
       <c r="H146" s="2" t="n">
-        <v>44.16242920524356</v>
+        <v>44.16242920348506</v>
       </c>
       <c r="I146" s="2" t="n">
-        <v>19.99641010840687</v>
+        <v>19.9964100552397</v>
       </c>
       <c r="J146" s="2" t="n">
         <v>0.6023231260713039</v>
@@ -8202,7 +8202,7 @@
         <v>-1</v>
       </c>
       <c r="N146" s="2" t="n">
-        <v>-0.3334610641080766</v>
+        <v>-0.333461064138987</v>
       </c>
       <c r="O146" s="2" t="inlineStr">
         <is>
@@ -8237,10 +8237,10 @@
         <v>0</v>
       </c>
       <c r="H147" s="2" t="n">
-        <v>47.64900016380813</v>
+        <v>47.64900009459809</v>
       </c>
       <c r="I147" s="2" t="n">
-        <v>17.71063169613414</v>
+        <v>17.71063186366871</v>
       </c>
       <c r="J147" s="2" t="n">
         <v>0.7147235516050578</v>
@@ -8255,7 +8255,7 @@
         <v>-1</v>
       </c>
       <c r="N147" s="2" t="n">
-        <v>0.0068654976970853</v>
+        <v>0.0068654977485961</v>
       </c>
       <c r="O147" s="2" t="inlineStr">
         <is>
@@ -8276,7 +8276,7 @@
         <v/>
       </c>
       <c r="D148" s="2" t="n">
-        <v>74.48547743959637</v>
+        <v>74.48547743959398</v>
       </c>
       <c r="E148" s="2" t="n">
         <v>25.7</v>
@@ -8290,10 +8290,10 @@
         <v>0</v>
       </c>
       <c r="H148" s="2" t="n">
-        <v>46.46610433308906</v>
+        <v>46.46610416286353</v>
       </c>
       <c r="I148" s="2" t="n">
-        <v>19.77013993243907</v>
+        <v>19.77013999688294</v>
       </c>
       <c r="J148" s="2" t="n">
         <v>0.5817551759240346</v>
@@ -8308,7 +8308,7 @@
         <v>-1</v>
       </c>
       <c r="N148" s="2" t="n">
-        <v>-0.1293239235208643</v>
+        <v>-0.1293239233251078</v>
       </c>
       <c r="O148" s="2" t="inlineStr">
         <is>

</xml_diff>